<commit_message>
Upgraded testing to Larger Scale of Simulations
Focus on improving accuracy of data by improving the number of trials, increasing the efficiency of the code and beginning to calculate the uncertainty that my tests fall within
</commit_message>
<xml_diff>
--- a/Flip 7 Data.xlsx
+++ b/Flip 7 Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b39dc15afb2f4832/Documents/Stuff/Github/Flip-7-Strategy-Finder/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3396" documentId="8_{518FECA9-5F80-4709-BD1F-73FC317A950E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9BE68D34-419E-4920-8A68-3CF9845029E8}"/>
+  <xr:revisionPtr revIDLastSave="3673" documentId="8_{518FECA9-5F80-4709-BD1F-73FC317A950E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{30C9B9ED-772E-47E0-85E3-322D0AFB8391}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{620B4B94-E82A-42AE-95A9-ED21412A2FCA}"/>
   </bookViews>
@@ -42,6 +42,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Master Data'!$C$62:$G$62</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -65,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1438" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1481" uniqueCount="259">
   <si>
     <t>Flip 7 Best Strat Test Data</t>
   </si>
@@ -725,6 +726,123 @@
   </si>
   <si>
     <t>These strategies are all similar efficiency but to take this testing further, I am going to need higher accuracy on the data to ensure that the correct conclusions are followed (prime example of this would be the misnomer that the score 30+ presented earlier in my testing). Therefore the number of trials I am doing for my chosen strategies is going to need to increase drastically and I think I've found a way to do that. For this set of tests I improved my effiency by making my code output the exact text I needed for the spreadsheet so that all I would need to do is copy the data in and excel would calculate it. If i want to scale my data up, I am not going to be able to record each score that is banked. So all data is going to have to remain in the python file. As a result of this I've decided that moving forward I will only need to post the results of my tests to the spreadsheet since I can run my game simulations in python and calculate the data values I'm using in the same file. So my next steps will be doing ~1 million simulations per strategy to try and get a good idea of the range of values that are best. In addition to this, I've also decided not to continue with the heuristics system for strategy testing as it is seeming to me that the score and probability methods are performing at a similar level and a human player can easily follow the score system without needing to complex calculations. So for my next (and likely final) set of tests I will test the values for score and probability around the 23 mark as that is what is seeming most optimal so far. Additionally I will be making some optimisations to the code to reduce some of the busts that the code is falling victim to that a human would avoid (namely banking as soon as 200 is reached and having this override the usual score or probabilty banking condition). So going forward, these are my newest goals to achieve.</t>
+  </si>
+  <si>
+    <t>Third set of strategies tested:</t>
+  </si>
+  <si>
+    <t>Always Bank (Score 20 +)</t>
+  </si>
+  <si>
+    <t>Always Bank (Score 21 +)</t>
+  </si>
+  <si>
+    <t>Always Bank (Score 22 +)</t>
+  </si>
+  <si>
+    <t>Always Bank (Score 23 +)</t>
+  </si>
+  <si>
+    <t>Always Bank (Score 24 +)</t>
+  </si>
+  <si>
+    <t>Always Bank (Score 25 +)</t>
+  </si>
+  <si>
+    <t>Always Bank (Score 26 +)</t>
+  </si>
+  <si>
+    <t>Average Total Score</t>
+  </si>
+  <si>
+    <t>Average Success Score</t>
+  </si>
+  <si>
+    <t>Unfortunately theres no data to link to here since there is just too much of it for me to be able to reasonably represent it on the spreadsheet (hence why only the results are shown here)</t>
+  </si>
+  <si>
+    <t>Always Bank (Score 27 +)</t>
+  </si>
+  <si>
+    <t>Always Bank (Score 28 +)</t>
+  </si>
+  <si>
+    <t>Always Bank (Score 29 +)</t>
+  </si>
+  <si>
+    <t>Always Bank (Score 30 +)</t>
+  </si>
+  <si>
+    <t>Always Bank (Score 31 +)</t>
+  </si>
+  <si>
+    <t>Always Bank (Score 32+)</t>
+  </si>
+  <si>
+    <t>Always Bank (Score 33+)</t>
+  </si>
+  <si>
+    <t>Always Bank (Score 34+)</t>
+  </si>
+  <si>
+    <t>Variability of Strategies:</t>
+  </si>
+  <si>
+    <t>Tested with Score 23+</t>
+  </si>
+  <si>
+    <t>Test 3</t>
+  </si>
+  <si>
+    <t>Test 4</t>
+  </si>
+  <si>
+    <t>Test 5</t>
+  </si>
+  <si>
+    <t>Test 6</t>
+  </si>
+  <si>
+    <t>Test 7</t>
+  </si>
+  <si>
+    <t>Test 8</t>
+  </si>
+  <si>
+    <t>Test 9</t>
+  </si>
+  <si>
+    <t>Test 10</t>
+  </si>
+  <si>
+    <t>Success vs Bust:</t>
+  </si>
+  <si>
+    <t>Mean:</t>
+  </si>
+  <si>
+    <t>Standard Deviation:</t>
+  </si>
+  <si>
+    <t>Uncertainty:</t>
+  </si>
+  <si>
+    <t>Results: (6 s.f)</t>
+  </si>
+  <si>
+    <t>204.913 ± 0.00481074</t>
+  </si>
+  <si>
+    <t>10.3033 ± 0.00124714</t>
+  </si>
+  <si>
+    <t>2.53611 ± 0.00115371</t>
+  </si>
+  <si>
+    <t>7.76830 ± 0.000382788</t>
+  </si>
+  <si>
+    <t>26.5153 ± 0.00127826</t>
   </si>
 </sst>
 </file>
@@ -3117,6 +3235,359 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-GB"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Master Data'!$E$173</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Average Rounds to 200</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Master Data'!$C$174:$C$188</c:f>
+              <c:strCache>
+                <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>Always Bank (Score 20 +)</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Always Bank (Score 21 +)</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Always Bank (Score 22 +)</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Always Bank (Score 23 +)</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Always Bank (Score 24 +)</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Always Bank (Score 25 +)</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Always Bank (Score 26 +)</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Always Bank (Score 27 +)</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Always Bank (Score 28 +)</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Always Bank (Score 29 +)</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Always Bank (Score 30 +)</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>Always Bank (Score 31 +)</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>Always Bank (Score 32+)</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>Always Bank (Score 33+)</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>Always Bank (Score 34+)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Master Data'!$E$174:$E$188</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>10.695829</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>10.532031</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>10.372769999999999</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>10.306252000000001</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>10.226029</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>10.118207999999999</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>10.109500000000001</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>10.168869000000001</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>10.235564</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>10.247678000000001</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>10.229124000000001</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>10.260602</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>10.400808</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>10.639106</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>10.911483</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-B09C-452B-A203-AA15391606A3}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="1482359951"/>
+        <c:axId val="1482361871"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1482359951"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1482361871"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1482361871"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1482359951"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -3198,6 +3669,46 @@
 </file>
 
 <file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors4.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -4785,6 +5296,509 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
@@ -4890,6 +5904,42 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>668365</xdr:colOff>
+      <xdr:row>188</xdr:row>
+      <xdr:rowOff>129798</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>857251</xdr:colOff>
+      <xdr:row>202</xdr:row>
+      <xdr:rowOff>160795</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="7" name="Chart 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EE0D0FBD-58B1-5534-417F-409128ADAD4E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -5471,14 +6521,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24461DB0-E066-4D80-9F31-EE0FB08E8CE2}">
-  <dimension ref="C2:CS202"/>
+  <dimension ref="C2:CS220"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="3" max="3" width="28.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="20.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="25.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="25.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="23.28515625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="18" bestFit="1" customWidth="1"/>
     <col min="10" max="11" width="20.7109375" bestFit="1" customWidth="1"/>
@@ -6896,23 +7945,23 @@
     </row>
     <row r="63" spans="3:15">
       <c r="C63" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="D63">
-        <f>'[1]Bank Score 23+'!AD103</f>
-        <v>9.81</v>
+        <f>'[1]Individual Odds 18%'!AD103</f>
+        <v>11.12</v>
       </c>
       <c r="E63">
-        <f>'[1]Bank Score 23+'!AE103</f>
-        <v>2.11</v>
+        <f>'[1]Individual Odds 18%'!AE103</f>
+        <v>2.27</v>
       </c>
       <c r="F63">
-        <f>'[1]Bank Score 23+'!AF103</f>
-        <v>7.7</v>
+        <f>'[1]Individual Odds 18%'!AF103</f>
+        <v>8.85</v>
       </c>
       <c r="G63">
-        <f>'[1]Bank Score 23+'!AG103</f>
-        <v>27.740297619047613</v>
+        <f>'[1]Individual Odds 18%'!AG103</f>
+        <v>24.296027417027421</v>
       </c>
       <c r="H63" s="4"/>
       <c r="I63" s="10" t="s">
@@ -6930,23 +7979,23 @@
     </row>
     <row r="64" spans="3:15">
       <c r="C64" t="s">
-        <v>208</v>
-      </c>
-      <c r="D64">
-        <f>'[1]Bank Score 22+'!AD103</f>
-        <v>10.3</v>
-      </c>
-      <c r="E64">
-        <f>'[1]Bank Score 22+'!AE103</f>
-        <v>2.2599999999999998</v>
-      </c>
-      <c r="F64">
-        <f>'[1]Bank Score 22+'!AF103</f>
-        <v>8.0399999999999991</v>
-      </c>
-      <c r="G64">
-        <f>'[1]Bank Score 22+'!AG103</f>
-        <v>26.516269841269835</v>
+        <v>43</v>
+      </c>
+      <c r="D64" s="2">
+        <f>'Bank Score 20+'!AD116</f>
+        <v>10.75</v>
+      </c>
+      <c r="E64" s="2">
+        <f>'Bank Score 20+'!AE116</f>
+        <v>2.0699999999999998</v>
+      </c>
+      <c r="F64" s="2">
+        <f>'Bank Score 20+'!AF116</f>
+        <v>8.68</v>
+      </c>
+      <c r="G64" s="2">
+        <f>'Bank Score 20+'!AG116</f>
+        <v>24.679059523809524</v>
       </c>
       <c r="H64" s="4"/>
       <c r="I64" s="10"/>
@@ -6962,23 +8011,23 @@
     </row>
     <row r="65" spans="3:15" ht="15" customHeight="1">
       <c r="C65" t="s">
-        <v>45</v>
+        <v>209</v>
       </c>
       <c r="D65">
-        <f>'Bank Score 30+'!AD116</f>
-        <v>10.3</v>
+        <f>'[1]Bank Score 21+'!AD103</f>
+        <v>10.46</v>
       </c>
       <c r="E65">
-        <f>'Bank Score 30+'!AE116</f>
-        <v>4.07</v>
+        <f>'[1]Bank Score 21+'!AE103</f>
+        <v>2.14</v>
       </c>
       <c r="F65">
-        <f>'Bank Score 30+'!AF116</f>
-        <v>6.23</v>
+        <f>'[1]Bank Score 21+'!AF103</f>
+        <v>8.32</v>
       </c>
       <c r="G65">
-        <f>'Bank Score 30+'!AG116</f>
-        <v>34.487333333333332</v>
+        <f>'[1]Bank Score 21+'!AG103</f>
+        <v>25.835992063492068</v>
       </c>
       <c r="H65" s="4"/>
       <c r="I65" s="10"/>
@@ -6994,23 +8043,23 @@
     </row>
     <row r="66" spans="3:15" ht="15" customHeight="1">
       <c r="C66" t="s">
-        <v>103</v>
+        <v>13</v>
       </c>
       <c r="D66">
-        <f>'[1]Bank Score 27+'!AD104</f>
-        <v>10.35</v>
+        <f>'Individual Odds 20%'!AD116</f>
+        <v>10.68</v>
       </c>
       <c r="E66">
-        <f>'[1]Bank Score 27+'!AE104</f>
-        <v>3.57</v>
+        <f>'Individual Odds 20%'!AE116</f>
+        <v>2.54</v>
       </c>
       <c r="F66">
-        <f>'[1]Bank Score 27+'!AF104</f>
-        <v>6.78</v>
+        <f>'Individual Odds 20%'!AF116</f>
+        <v>8.14</v>
       </c>
       <c r="G66">
-        <f>'[1]Bank Score 27+'!AG104</f>
-        <v>32.142559523809524</v>
+        <f>'Individual Odds 20%'!AG116</f>
+        <v>26.310999999999993</v>
       </c>
       <c r="H66" s="4"/>
       <c r="I66" s="10"/>
@@ -7026,23 +8075,23 @@
     </row>
     <row r="67" spans="3:15" ht="15" customHeight="1">
       <c r="C67" t="s">
-        <v>112</v>
+        <v>208</v>
       </c>
       <c r="D67">
-        <f>'[1]Bank Score 24+'!AD103</f>
-        <v>10.42</v>
+        <f>'[1]Bank Score 22+'!AD103</f>
+        <v>10.3</v>
       </c>
       <c r="E67">
-        <f>'[1]Bank Score 24+'!AE103</f>
-        <v>2.95</v>
+        <f>'[1]Bank Score 22+'!AE103</f>
+        <v>2.2599999999999998</v>
       </c>
       <c r="F67">
-        <f>'[1]Bank Score 24+'!AF103</f>
-        <v>7.47</v>
+        <f>'[1]Bank Score 22+'!AF103</f>
+        <v>8.0399999999999991</v>
       </c>
       <c r="G67">
-        <f>'[1]Bank Score 24+'!AG103</f>
-        <v>28.778928571428573</v>
+        <f>'[1]Bank Score 22+'!AG103</f>
+        <v>26.516269841269835</v>
       </c>
       <c r="H67" s="4"/>
       <c r="I67" s="10"/>
@@ -7058,23 +8107,23 @@
     </row>
     <row r="68" spans="3:15">
       <c r="C68" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D68">
-        <f>'[1]Bank Score 26+'!AD103</f>
-        <v>10.44</v>
+        <f>'[1]Bank Score 23+'!AD103</f>
+        <v>9.81</v>
       </c>
       <c r="E68">
-        <f>'[1]Bank Score 26+'!AE103</f>
-        <v>3.49</v>
+        <f>'[1]Bank Score 23+'!AE103</f>
+        <v>2.11</v>
       </c>
       <c r="F68">
-        <f>'[1]Bank Score 26+'!AF103</f>
-        <v>6.95</v>
+        <f>'[1]Bank Score 23+'!AF103</f>
+        <v>7.7</v>
       </c>
       <c r="G68">
-        <f>'[1]Bank Score 26+'!AG103</f>
-        <v>30.939047619047614</v>
+        <f>'[1]Bank Score 23+'!AG103</f>
+        <v>27.740297619047613</v>
       </c>
       <c r="H68" s="4"/>
       <c r="I68" s="10"/>
@@ -7090,23 +8139,23 @@
     </row>
     <row r="69" spans="3:15">
       <c r="C69" t="s">
-        <v>209</v>
+        <v>107</v>
       </c>
       <c r="D69">
-        <f>'[1]Bank Score 21+'!AD103</f>
-        <v>10.46</v>
+        <f>'[1]Individual Odds 22%'!AD103</f>
+        <v>10.52</v>
       </c>
       <c r="E69">
-        <f>'[1]Bank Score 21+'!AE103</f>
-        <v>2.14</v>
+        <f>'[1]Individual Odds 22%'!AE103</f>
+        <v>2.82</v>
       </c>
       <c r="F69">
-        <f>'[1]Bank Score 21+'!AF103</f>
-        <v>8.32</v>
+        <f>'[1]Individual Odds 22%'!AF103</f>
+        <v>7.7</v>
       </c>
       <c r="G69">
-        <f>'[1]Bank Score 21+'!AG103</f>
-        <v>25.835992063492068</v>
+        <f>'[1]Individual Odds 22%'!AG103</f>
+        <v>28.177678571428572</v>
       </c>
       <c r="H69" s="4"/>
       <c r="I69" s="10"/>
@@ -7122,23 +8171,23 @@
     </row>
     <row r="70" spans="3:15">
       <c r="C70" t="s">
-        <v>44</v>
+        <v>112</v>
       </c>
       <c r="D70">
-        <f>'Bank Score 25+'!AD116</f>
-        <v>10.46</v>
+        <f>'[1]Bank Score 24+'!AD103</f>
+        <v>10.42</v>
       </c>
       <c r="E70">
-        <f>'Bank Score 25+'!AE116</f>
-        <v>3.32</v>
+        <f>'[1]Bank Score 24+'!AE103</f>
+        <v>2.95</v>
       </c>
       <c r="F70">
-        <f>'Bank Score 25+'!AF116</f>
-        <v>7.14</v>
+        <f>'[1]Bank Score 24+'!AF103</f>
+        <v>7.47</v>
       </c>
       <c r="G70">
-        <f>'Bank Score 25+'!AG116</f>
-        <v>29.96363095238096</v>
+        <f>'[1]Bank Score 24+'!AG103</f>
+        <v>28.778928571428573</v>
       </c>
       <c r="H70" s="4"/>
       <c r="I70" s="6"/>
@@ -7154,23 +8203,23 @@
     </row>
     <row r="71" spans="3:15">
       <c r="C71" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D71">
-        <f>'[1]Individual Odds 22%'!AD103</f>
-        <v>10.52</v>
+        <f>'[1]Individual Odds 24%'!AD103</f>
+        <v>10.94</v>
       </c>
       <c r="E71">
-        <f>'[1]Individual Odds 22%'!AE103</f>
-        <v>2.82</v>
+        <f>'[1]Individual Odds 24%'!AE103</f>
+        <v>3.72</v>
       </c>
       <c r="F71">
-        <f>'[1]Individual Odds 22%'!AF103</f>
-        <v>7.7</v>
+        <f>'[1]Individual Odds 24%'!AF103</f>
+        <v>7.22</v>
       </c>
       <c r="G71">
-        <f>'[1]Individual Odds 22%'!AG103</f>
-        <v>28.177678571428572</v>
+        <f>'[1]Individual Odds 24%'!AG103</f>
+        <v>30.149138888888888</v>
       </c>
       <c r="H71" s="4"/>
       <c r="I71" s="6"/>
@@ -7186,23 +8235,23 @@
     </row>
     <row r="72" spans="3:15">
       <c r="C72" t="s">
-        <v>109</v>
+        <v>44</v>
       </c>
       <c r="D72">
-        <f>'[1]Individual Odds 26%'!AD103</f>
-        <v>10.55</v>
+        <f>'Bank Score 25+'!AD116</f>
+        <v>10.46</v>
       </c>
       <c r="E72">
-        <f>'[1]Individual Odds 26%'!AE103</f>
-        <v>3.77</v>
+        <f>'Bank Score 25+'!AE116</f>
+        <v>3.32</v>
       </c>
       <c r="F72">
-        <f>'[1]Individual Odds 26%'!AF103</f>
-        <v>6.78</v>
+        <f>'Bank Score 25+'!AF116</f>
+        <v>7.14</v>
       </c>
       <c r="G72">
-        <f>'[1]Individual Odds 26%'!AG103</f>
-        <v>32.079047619047621</v>
+        <f>'Bank Score 25+'!AG116</f>
+        <v>29.96363095238096</v>
       </c>
       <c r="H72" s="4"/>
       <c r="K72">
@@ -7217,23 +8266,23 @@
     </row>
     <row r="73" spans="3:15">
       <c r="C73" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="D73">
-        <f>'[1]Bank Score 28+'!AD104</f>
-        <v>10.67</v>
+        <f>'[1]Bank Score 26+'!AD103</f>
+        <v>10.44</v>
       </c>
       <c r="E73">
-        <f>'[1]Bank Score 28+'!AE104</f>
-        <v>3.95</v>
+        <f>'[1]Bank Score 26+'!AE103</f>
+        <v>3.49</v>
       </c>
       <c r="F73">
-        <f>'[1]Bank Score 28+'!AF104</f>
-        <v>6.72</v>
+        <f>'[1]Bank Score 26+'!AF103</f>
+        <v>6.95</v>
       </c>
       <c r="G73">
-        <f>'[1]Bank Score 28+'!AG104</f>
-        <v>32.876904761904761</v>
+        <f>'[1]Bank Score 26+'!AG103</f>
+        <v>30.939047619047614</v>
       </c>
       <c r="H73" s="4"/>
       <c r="K73">
@@ -7248,23 +8297,23 @@
     </row>
     <row r="74" spans="3:15">
       <c r="C74" t="s">
-        <v>13</v>
+        <v>103</v>
       </c>
       <c r="D74">
-        <f>'Individual Odds 20%'!AD116</f>
-        <v>10.68</v>
+        <f>'[1]Bank Score 27+'!AD104</f>
+        <v>10.35</v>
       </c>
       <c r="E74">
-        <f>'Individual Odds 20%'!AE116</f>
-        <v>2.54</v>
+        <f>'[1]Bank Score 27+'!AE104</f>
+        <v>3.57</v>
       </c>
       <c r="F74">
-        <f>'Individual Odds 20%'!AF116</f>
-        <v>8.14</v>
+        <f>'[1]Bank Score 27+'!AF104</f>
+        <v>6.78</v>
       </c>
       <c r="G74">
-        <f>'Individual Odds 20%'!AG116</f>
-        <v>26.310999999999993</v>
+        <f>'[1]Bank Score 27+'!AG104</f>
+        <v>32.142559523809524</v>
       </c>
       <c r="H74" s="4"/>
       <c r="K74">
@@ -7279,23 +8328,23 @@
     </row>
     <row r="75" spans="3:15">
       <c r="C75" t="s">
-        <v>43</v>
-      </c>
-      <c r="D75" s="2">
-        <f>'Bank Score 20+'!AD116</f>
-        <v>10.75</v>
-      </c>
-      <c r="E75" s="2">
-        <f>'Bank Score 20+'!AE116</f>
-        <v>2.0699999999999998</v>
-      </c>
-      <c r="F75" s="2">
-        <f>'Bank Score 20+'!AF116</f>
-        <v>8.68</v>
-      </c>
-      <c r="G75" s="2">
-        <f>'Bank Score 20+'!AG116</f>
-        <v>24.679059523809524</v>
+        <v>109</v>
+      </c>
+      <c r="D75">
+        <f>'[1]Individual Odds 26%'!AD103</f>
+        <v>10.55</v>
+      </c>
+      <c r="E75">
+        <f>'[1]Individual Odds 26%'!AE103</f>
+        <v>3.77</v>
+      </c>
+      <c r="F75">
+        <f>'[1]Individual Odds 26%'!AF103</f>
+        <v>6.78</v>
+      </c>
+      <c r="G75">
+        <f>'[1]Individual Odds 26%'!AG103</f>
+        <v>32.079047619047621</v>
       </c>
       <c r="H75" s="4"/>
       <c r="K75">
@@ -7310,23 +8359,23 @@
     </row>
     <row r="76" spans="3:15">
       <c r="C76" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="D76">
-        <f>'[1]Individual Odds 28%'!AD103</f>
-        <v>10.76</v>
+        <f>'[1]Bank Score 28+'!AD104</f>
+        <v>10.67</v>
       </c>
       <c r="E76">
-        <f>'[1]Individual Odds 28%'!AE103</f>
-        <v>4.38</v>
+        <f>'[1]Bank Score 28+'!AE104</f>
+        <v>3.95</v>
       </c>
       <c r="F76">
-        <f>'[1]Individual Odds 28%'!AF103</f>
-        <v>6.38</v>
+        <f>'[1]Bank Score 28+'!AF104</f>
+        <v>6.72</v>
       </c>
       <c r="G76">
-        <f>'[1]Individual Odds 28%'!AG103</f>
-        <v>34.557734126984116</v>
+        <f>'[1]Bank Score 28+'!AG104</f>
+        <v>32.876904761904761</v>
       </c>
       <c r="H76" s="4"/>
       <c r="K76">
@@ -7341,23 +8390,23 @@
     </row>
     <row r="77" spans="3:15">
       <c r="C77" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="D77">
-        <f>'[1]Individual Odds 24%'!AD103</f>
-        <v>10.94</v>
+        <f>'[1]Bank Score 29+'!AD103</f>
+        <v>11.19</v>
       </c>
       <c r="E77">
-        <f>'[1]Individual Odds 24%'!AE103</f>
-        <v>3.72</v>
+        <f>'[1]Bank Score 29+'!AE103</f>
+        <v>4.7300000000000004</v>
       </c>
       <c r="F77">
-        <f>'[1]Individual Odds 24%'!AF103</f>
-        <v>7.22</v>
+        <f>'[1]Bank Score 29+'!AF103</f>
+        <v>6.46</v>
       </c>
       <c r="G77">
-        <f>'[1]Individual Odds 24%'!AG103</f>
-        <v>30.149138888888888</v>
+        <f>'[1]Bank Score 29+'!AG103</f>
+        <v>33.759904761904764</v>
       </c>
       <c r="H77" s="4"/>
       <c r="K77">
@@ -7372,23 +8421,23 @@
     </row>
     <row r="78" spans="3:15">
       <c r="C78" t="s">
-        <v>14</v>
+        <v>110</v>
       </c>
       <c r="D78">
-        <f>'Individual Odds 30%'!AD116</f>
-        <v>11.02</v>
+        <f>'[1]Individual Odds 28%'!AD103</f>
+        <v>10.76</v>
       </c>
       <c r="E78">
-        <f>'Individual Odds 30%'!AE116</f>
-        <v>4.9400000000000004</v>
+        <f>'[1]Individual Odds 28%'!AE103</f>
+        <v>4.38</v>
       </c>
       <c r="F78">
-        <f>'Individual Odds 30%'!AF116</f>
-        <v>6.08</v>
+        <f>'[1]Individual Odds 28%'!AF103</f>
+        <v>6.38</v>
       </c>
       <c r="G78">
-        <f>'Individual Odds 30%'!AG116</f>
-        <v>36.181940476190469</v>
+        <f>'[1]Individual Odds 28%'!AG103</f>
+        <v>34.557734126984116</v>
       </c>
       <c r="H78" s="4"/>
       <c r="K78">
@@ -7403,23 +8452,23 @@
     </row>
     <row r="79" spans="3:15">
       <c r="C79" t="s">
-        <v>106</v>
+        <v>45</v>
       </c>
       <c r="D79">
-        <f>'[1]Individual Odds 18%'!AD103</f>
-        <v>11.12</v>
+        <f>'Bank Score 30+'!AD116</f>
+        <v>10.3</v>
       </c>
       <c r="E79">
-        <f>'[1]Individual Odds 18%'!AE103</f>
-        <v>2.27</v>
+        <f>'Bank Score 30+'!AE116</f>
+        <v>4.07</v>
       </c>
       <c r="F79">
-        <f>'[1]Individual Odds 18%'!AF103</f>
-        <v>8.85</v>
+        <f>'Bank Score 30+'!AF116</f>
+        <v>6.23</v>
       </c>
       <c r="G79">
-        <f>'[1]Individual Odds 18%'!AG103</f>
-        <v>24.296027417027421</v>
+        <f>'Bank Score 30+'!AG116</f>
+        <v>34.487333333333332</v>
       </c>
       <c r="H79" s="4"/>
       <c r="K79">
@@ -7434,23 +8483,23 @@
     </row>
     <row r="80" spans="3:15">
       <c r="C80" t="s">
-        <v>105</v>
+        <v>14</v>
       </c>
       <c r="D80">
-        <f>'[1]Bank Score 29+'!AD103</f>
-        <v>11.19</v>
+        <f>'Individual Odds 30%'!AD116</f>
+        <v>11.02</v>
       </c>
       <c r="E80">
-        <f>'[1]Bank Score 29+'!AE103</f>
-        <v>4.7300000000000004</v>
+        <f>'Individual Odds 30%'!AE116</f>
+        <v>4.9400000000000004</v>
       </c>
       <c r="F80">
-        <f>'[1]Bank Score 29+'!AF103</f>
-        <v>6.46</v>
+        <f>'Individual Odds 30%'!AF116</f>
+        <v>6.08</v>
       </c>
       <c r="G80">
-        <f>'[1]Bank Score 29+'!AG103</f>
-        <v>33.759904761904764</v>
+        <f>'Individual Odds 30%'!AG116</f>
+        <v>36.181940476190469</v>
       </c>
       <c r="H80" s="4"/>
       <c r="K80">
@@ -7985,160 +9034,812 @@
     <row r="160" spans="3:3">
       <c r="C160" s="8"/>
     </row>
-    <row r="161" spans="3:8">
+    <row r="161" spans="3:10">
       <c r="C161" s="8"/>
     </row>
-    <row r="162" spans="3:8">
+    <row r="162" spans="3:10">
       <c r="C162" s="8"/>
     </row>
-    <row r="163" spans="3:8">
+    <row r="163" spans="3:10">
       <c r="C163" s="8"/>
     </row>
-    <row r="164" spans="3:8">
+    <row r="164" spans="3:10">
       <c r="C164" s="8"/>
     </row>
-    <row r="165" spans="3:8">
+    <row r="165" spans="3:10">
       <c r="C165" s="8"/>
     </row>
-    <row r="166" spans="3:8">
+    <row r="166" spans="3:10">
       <c r="C166" s="8"/>
     </row>
-    <row r="167" spans="3:8">
+    <row r="167" spans="3:10">
       <c r="C167" s="8"/>
     </row>
-    <row r="168" spans="3:8">
+    <row r="168" spans="3:10">
       <c r="C168" s="8"/>
     </row>
-    <row r="169" spans="3:8">
+    <row r="169" spans="3:10">
       <c r="C169" s="8"/>
     </row>
-    <row r="170" spans="3:8">
+    <row r="170" spans="3:10">
       <c r="C170" s="8"/>
     </row>
-    <row r="171" spans="3:8">
+    <row r="171" spans="3:10">
       <c r="C171" s="7"/>
     </row>
-    <row r="172" spans="3:8">
+    <row r="172" spans="3:10">
       <c r="C172" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="173" spans="3:8">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="173" spans="3:10">
       <c r="D173" t="s">
+        <v>228</v>
+      </c>
+      <c r="E173" t="s">
         <v>10</v>
       </c>
-      <c r="E173" t="s">
+      <c r="F173" t="s">
         <v>79</v>
       </c>
-      <c r="F173" t="s">
+      <c r="G173" t="s">
         <v>78</v>
       </c>
-      <c r="G173" t="s">
-        <v>77</v>
-      </c>
       <c r="H173" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="174" spans="3:8">
-      <c r="C174" s="7"/>
-    </row>
-    <row r="175" spans="3:8">
-      <c r="C175" s="7"/>
-    </row>
-    <row r="176" spans="3:8">
-      <c r="C176" s="7"/>
-    </row>
-    <row r="177" spans="3:3">
-      <c r="C177" s="7"/>
-    </row>
-    <row r="178" spans="3:3">
-      <c r="C178" s="7"/>
-    </row>
-    <row r="179" spans="3:3">
-      <c r="C179" s="7"/>
-    </row>
-    <row r="180" spans="3:3">
-      <c r="C180" s="7"/>
-    </row>
-    <row r="181" spans="3:3">
-      <c r="C181" s="7"/>
-    </row>
-    <row r="182" spans="3:3">
-      <c r="C182" s="7"/>
-    </row>
-    <row r="183" spans="3:3">
-      <c r="C183" s="7"/>
-    </row>
-    <row r="184" spans="3:3">
-      <c r="C184" s="7"/>
-    </row>
-    <row r="185" spans="3:3">
-      <c r="C185" s="7"/>
-    </row>
-    <row r="186" spans="3:3">
-      <c r="C186" s="7"/>
-    </row>
-    <row r="187" spans="3:3">
-      <c r="C187" s="7"/>
-    </row>
-    <row r="188" spans="3:3">
-      <c r="C188" s="7"/>
-    </row>
-    <row r="189" spans="3:3">
+        <v>229</v>
+      </c>
+      <c r="I173" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="174" spans="3:10" ht="15" customHeight="1">
+      <c r="C174" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="D174">
+        <v>204.928854</v>
+      </c>
+      <c r="E174">
+        <v>10.695829</v>
+      </c>
+      <c r="F174">
+        <v>2.0003600000000001</v>
+      </c>
+      <c r="G174">
+        <v>8.6954689999999992</v>
+      </c>
+      <c r="H174">
+        <v>23.6955327936281</v>
+      </c>
+      <c r="I174">
+        <f>G174/F174</f>
+        <v>4.3469520486312456</v>
+      </c>
+      <c r="J174" s="9" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="175" spans="3:10">
+      <c r="C175" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="D175">
+        <v>204.92634200000001</v>
+      </c>
+      <c r="E175">
+        <v>10.532031</v>
+      </c>
+      <c r="F175">
+        <v>2.166674</v>
+      </c>
+      <c r="G175">
+        <v>8.3653569999999995</v>
+      </c>
+      <c r="H175">
+        <v>24.641126278171399</v>
+      </c>
+      <c r="I175">
+        <f t="shared" ref="I175:I188" si="0">G175/F175</f>
+        <v>3.8609209322676135</v>
+      </c>
+      <c r="J175" s="9"/>
+    </row>
+    <row r="176" spans="3:10">
+      <c r="C176" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="D176">
+        <v>204.90937299999999</v>
+      </c>
+      <c r="E176">
+        <v>10.372769999999999</v>
+      </c>
+      <c r="F176">
+        <v>2.3642599999999998</v>
+      </c>
+      <c r="G176">
+        <v>8.0085099999999994</v>
+      </c>
+      <c r="H176">
+        <v>25.710231051580699</v>
+      </c>
+      <c r="I176">
+        <f t="shared" si="0"/>
+        <v>3.3873220373393789</v>
+      </c>
+      <c r="J176" s="9"/>
+    </row>
+    <row r="177" spans="3:10">
+      <c r="C177" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="D177">
+        <v>204.90204800000001</v>
+      </c>
+      <c r="E177">
+        <v>10.306252000000001</v>
+      </c>
+      <c r="F177">
+        <v>2.5378090000000002</v>
+      </c>
+      <c r="G177">
+        <v>7.7684430000000004</v>
+      </c>
+      <c r="H177">
+        <v>26.514071702364198</v>
+      </c>
+      <c r="I177">
+        <f t="shared" si="0"/>
+        <v>3.0610826110239184</v>
+      </c>
+      <c r="J177" s="9"/>
+    </row>
+    <row r="178" spans="3:10">
+      <c r="C178" s="7" t="s">
+        <v>225</v>
+      </c>
+      <c r="D178">
+        <v>204.90852699999999</v>
+      </c>
+      <c r="E178">
+        <v>10.226029</v>
+      </c>
+      <c r="F178">
+        <v>2.7698559999999999</v>
+      </c>
+      <c r="G178">
+        <v>7.4561729999999997</v>
+      </c>
+      <c r="H178">
+        <v>27.661426526549299</v>
+      </c>
+      <c r="I178">
+        <f t="shared" si="0"/>
+        <v>2.6918991456595576</v>
+      </c>
+      <c r="J178" s="9"/>
+    </row>
+    <row r="179" spans="3:10">
+      <c r="C179" s="7" t="s">
+        <v>226</v>
+      </c>
+      <c r="D179">
+        <v>204.87778700000001</v>
+      </c>
+      <c r="E179">
+        <v>10.118207999999999</v>
+      </c>
+      <c r="F179">
+        <v>2.9605100000000002</v>
+      </c>
+      <c r="G179">
+        <v>7.1576979999999999</v>
+      </c>
+      <c r="H179">
+        <v>28.770401677324799</v>
+      </c>
+      <c r="I179">
+        <f t="shared" si="0"/>
+        <v>2.4177246487936199</v>
+      </c>
+      <c r="J179" s="9"/>
+    </row>
+    <row r="180" spans="3:10">
+      <c r="C180" s="7" t="s">
+        <v>227</v>
+      </c>
+      <c r="D180">
+        <v>204.84169800000001</v>
+      </c>
+      <c r="E180">
+        <v>10.109500000000001</v>
+      </c>
+      <c r="F180">
+        <v>3.1620550000000001</v>
+      </c>
+      <c r="G180">
+        <v>6.9474450000000001</v>
+      </c>
+      <c r="H180">
+        <v>29.576063808268401</v>
+      </c>
+      <c r="I180">
+        <f t="shared" si="0"/>
+        <v>2.1971297146950324</v>
+      </c>
+      <c r="J180" s="9"/>
+    </row>
+    <row r="181" spans="3:10">
+      <c r="C181" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="D181">
+        <v>204.881719</v>
+      </c>
+      <c r="E181">
+        <v>10.168869000000001</v>
+      </c>
+      <c r="F181">
+        <v>3.3134250000000001</v>
+      </c>
+      <c r="G181">
+        <v>6.8554440000000003</v>
+      </c>
+      <c r="H181">
+        <v>29.997730984461601</v>
+      </c>
+      <c r="I181">
+        <f t="shared" si="0"/>
+        <v>2.0689902442336856</v>
+      </c>
+      <c r="J181" s="9"/>
+    </row>
+    <row r="182" spans="3:10">
+      <c r="C182" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="D182">
+        <v>204.924961</v>
+      </c>
+      <c r="E182">
+        <v>10.235564</v>
+      </c>
+      <c r="F182">
+        <v>3.5172870000000001</v>
+      </c>
+      <c r="G182">
+        <v>6.7182769999999996</v>
+      </c>
+      <c r="H182">
+        <v>30.680995797563401</v>
+      </c>
+      <c r="I182">
+        <f t="shared" si="0"/>
+        <v>1.9100735879670894</v>
+      </c>
+      <c r="J182" s="9"/>
+    </row>
+    <row r="183" spans="3:10">
+      <c r="C183" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="D183">
+        <v>204.917868</v>
+      </c>
+      <c r="E183">
+        <v>10.247678000000001</v>
+      </c>
+      <c r="F183">
+        <v>3.7666819999999999</v>
+      </c>
+      <c r="G183">
+        <v>6.4809960000000002</v>
+      </c>
+      <c r="H183">
+        <v>31.856338171378201</v>
+      </c>
+      <c r="I183">
+        <f t="shared" si="0"/>
+        <v>1.7206114028208381</v>
+      </c>
+      <c r="J183" s="9"/>
+    </row>
+    <row r="184" spans="3:10">
+      <c r="C184" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="D184">
+        <v>204.86341999999999</v>
+      </c>
+      <c r="E184">
+        <v>10.229124000000001</v>
+      </c>
+      <c r="F184">
+        <v>4.0175130000000001</v>
+      </c>
+      <c r="G184">
+        <v>6.2116110000000004</v>
+      </c>
+      <c r="H184">
+        <v>33.190480828526397</v>
+      </c>
+      <c r="I184">
+        <f t="shared" si="0"/>
+        <v>1.5461333914787583</v>
+      </c>
+    </row>
+    <row r="185" spans="3:10">
+      <c r="C185" s="7" t="s">
+        <v>235</v>
+      </c>
+      <c r="D185">
+        <v>204.792878</v>
+      </c>
+      <c r="E185">
+        <v>10.260602</v>
+      </c>
+      <c r="F185">
+        <v>4.2541520000000004</v>
+      </c>
+      <c r="G185">
+        <v>6.0064500000000001</v>
+      </c>
+      <c r="H185">
+        <v>34.217799095202501</v>
+      </c>
+      <c r="I185">
+        <f t="shared" si="0"/>
+        <v>1.4119030067566931</v>
+      </c>
+    </row>
+    <row r="186" spans="3:10">
+      <c r="C186" s="7" t="s">
+        <v>236</v>
+      </c>
+      <c r="D186">
+        <v>204.78541200000001</v>
+      </c>
+      <c r="E186">
+        <v>10.400808</v>
+      </c>
+      <c r="F186">
+        <v>4.4751450000000004</v>
+      </c>
+      <c r="G186">
+        <v>5.9256630000000001</v>
+      </c>
+      <c r="H186">
+        <v>34.654331254727502</v>
+      </c>
+      <c r="I186">
+        <f t="shared" si="0"/>
+        <v>1.3241275981001732</v>
+      </c>
+    </row>
+    <row r="187" spans="3:10">
+      <c r="C187" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="D187">
+        <v>204.82618600000001</v>
+      </c>
+      <c r="E187">
+        <v>10.639106</v>
+      </c>
+      <c r="F187">
+        <v>4.7586120000000003</v>
+      </c>
+      <c r="G187">
+        <v>5.8804939999999997</v>
+      </c>
+      <c r="H187">
+        <v>34.957205602348502</v>
+      </c>
+      <c r="I187">
+        <f t="shared" si="0"/>
+        <v>1.2357582421092537</v>
+      </c>
+    </row>
+    <row r="188" spans="3:10">
+      <c r="C188" s="7" t="s">
+        <v>238</v>
+      </c>
+      <c r="D188">
+        <v>204.91319300000001</v>
+      </c>
+      <c r="E188">
+        <v>10.911483</v>
+      </c>
+      <c r="F188">
+        <v>5.1167769999999999</v>
+      </c>
+      <c r="G188">
+        <v>5.7947059999999997</v>
+      </c>
+      <c r="H188">
+        <v>35.557773966639303</v>
+      </c>
+      <c r="I188">
+        <f t="shared" si="0"/>
+        <v>1.1324914101200814</v>
+      </c>
+    </row>
+    <row r="189" spans="3:10">
       <c r="C189" s="7"/>
     </row>
-    <row r="190" spans="3:3">
+    <row r="190" spans="3:10">
       <c r="C190" s="7"/>
     </row>
-    <row r="191" spans="3:3">
+    <row r="191" spans="3:10">
       <c r="C191" s="7"/>
     </row>
-    <row r="192" spans="3:3">
+    <row r="192" spans="3:10">
       <c r="C192" s="7"/>
     </row>
-    <row r="193" spans="3:3">
+    <row r="193" spans="3:8">
       <c r="C193" s="7"/>
     </row>
-    <row r="194" spans="3:3">
+    <row r="194" spans="3:8">
       <c r="C194" s="7"/>
     </row>
-    <row r="195" spans="3:3">
+    <row r="195" spans="3:8">
       <c r="C195" s="7"/>
     </row>
-    <row r="196" spans="3:3">
+    <row r="196" spans="3:8">
       <c r="C196" s="7"/>
     </row>
-    <row r="197" spans="3:3">
+    <row r="197" spans="3:8">
       <c r="C197" s="7"/>
     </row>
-    <row r="198" spans="3:3">
+    <row r="198" spans="3:8">
       <c r="C198" s="7"/>
     </row>
-    <row r="199" spans="3:3">
+    <row r="199" spans="3:8">
       <c r="C199" s="7"/>
     </row>
-    <row r="200" spans="3:3">
+    <row r="200" spans="3:8">
       <c r="C200" s="7"/>
     </row>
-    <row r="201" spans="3:3">
+    <row r="201" spans="3:8">
       <c r="C201" s="7"/>
     </row>
-    <row r="202" spans="3:3">
+    <row r="202" spans="3:8">
       <c r="C202" s="7"/>
+    </row>
+    <row r="204" spans="3:8">
+      <c r="C204" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="205" spans="3:8">
+      <c r="C205" t="s">
+        <v>240</v>
+      </c>
+      <c r="D205" t="s">
+        <v>228</v>
+      </c>
+      <c r="E205" t="s">
+        <v>10</v>
+      </c>
+      <c r="F205" t="s">
+        <v>79</v>
+      </c>
+      <c r="G205" t="s">
+        <v>78</v>
+      </c>
+      <c r="H205" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="206" spans="3:8">
+      <c r="C206" t="s">
+        <v>98</v>
+      </c>
+      <c r="D206">
+        <v>204.91085899999999</v>
+      </c>
+      <c r="E206">
+        <v>10.304460000000001</v>
+      </c>
+      <c r="F206">
+        <v>2.5366719999999998</v>
+      </c>
+      <c r="G206">
+        <v>7.7677880000000004</v>
+      </c>
+      <c r="H206">
+        <v>26.517588402760602</v>
+      </c>
+    </row>
+    <row r="207" spans="3:8">
+      <c r="C207" t="s">
+        <v>99</v>
+      </c>
+      <c r="D207">
+        <v>204.903502</v>
+      </c>
+      <c r="E207">
+        <v>10.302578</v>
+      </c>
+      <c r="F207">
+        <v>2.5344069999999999</v>
+      </c>
+      <c r="G207">
+        <v>7.7681709999999997</v>
+      </c>
+      <c r="H207">
+        <v>26.5150712404591</v>
+      </c>
+    </row>
+    <row r="208" spans="3:8">
+      <c r="C208" t="s">
+        <v>241</v>
+      </c>
+      <c r="D208">
+        <v>204.909357</v>
+      </c>
+      <c r="E208">
+        <v>10.30499</v>
+      </c>
+      <c r="F208">
+        <v>2.5371700000000001</v>
+      </c>
+      <c r="G208">
+        <v>7.7678200000000004</v>
+      </c>
+      <c r="H208">
+        <v>26.5174803110935</v>
+      </c>
+    </row>
+    <row r="209" spans="3:8">
+      <c r="C209" t="s">
+        <v>242</v>
+      </c>
+      <c r="D209">
+        <v>204.91343000000001</v>
+      </c>
+      <c r="E209">
+        <v>10.305558</v>
+      </c>
+      <c r="F209">
+        <v>2.5364089999999999</v>
+      </c>
+      <c r="G209">
+        <v>7.7691489999999996</v>
+      </c>
+      <c r="H209">
+        <v>26.512915067443501</v>
+      </c>
+    </row>
+    <row r="210" spans="3:8">
+      <c r="C210" t="s">
+        <v>243</v>
+      </c>
+      <c r="D210">
+        <v>204.916573</v>
+      </c>
+      <c r="E210">
+        <v>10.304254999999999</v>
+      </c>
+      <c r="F210">
+        <v>2.535622</v>
+      </c>
+      <c r="G210">
+        <v>7.7686330000000003</v>
+      </c>
+      <c r="H210">
+        <v>26.5151773761737</v>
+      </c>
+    </row>
+    <row r="211" spans="3:8">
+      <c r="C211" t="s">
+        <v>244</v>
+      </c>
+      <c r="D211">
+        <v>204.91018700000001</v>
+      </c>
+      <c r="E211">
+        <v>10.307034</v>
+      </c>
+      <c r="F211">
+        <v>2.5380929999999999</v>
+      </c>
+      <c r="G211">
+        <v>7.7689409999999999</v>
+      </c>
+      <c r="H211">
+        <v>26.5129467511737</v>
+      </c>
+    </row>
+    <row r="212" spans="3:8">
+      <c r="C212" t="s">
+        <v>245</v>
+      </c>
+      <c r="D212">
+        <v>204.89928499999999</v>
+      </c>
+      <c r="E212">
+        <v>10.304995999999999</v>
+      </c>
+      <c r="F212">
+        <v>2.5369739999999998</v>
+      </c>
+      <c r="G212">
+        <v>7.7680220000000002</v>
+      </c>
+      <c r="H212">
+        <v>26.514916359506898</v>
+      </c>
+    </row>
+    <row r="213" spans="3:8">
+      <c r="C213" t="s">
+        <v>246</v>
+      </c>
+      <c r="D213">
+        <v>204.899507</v>
+      </c>
+      <c r="E213">
+        <v>10.302797999999999</v>
+      </c>
+      <c r="F213">
+        <v>2.5348440000000001</v>
+      </c>
+      <c r="G213">
+        <v>7.7679539999999996</v>
+      </c>
+      <c r="H213">
+        <v>26.5153890618875</v>
+      </c>
+    </row>
+    <row r="214" spans="3:8">
+      <c r="C214" t="s">
+        <v>247</v>
+      </c>
+      <c r="D214">
+        <v>204.91061999999999</v>
+      </c>
+      <c r="E214">
+        <v>10.305367</v>
+      </c>
+      <c r="F214">
+        <v>2.5372279999999998</v>
+      </c>
+      <c r="G214">
+        <v>7.7681389999999997</v>
+      </c>
+      <c r="H214">
+        <v>26.516137601967198</v>
+      </c>
+    </row>
+    <row r="215" spans="3:8">
+      <c r="C215" t="s">
+        <v>248</v>
+      </c>
+      <c r="D215">
+        <v>204.91299599999999</v>
+      </c>
+      <c r="E215">
+        <v>10.302104</v>
+      </c>
+      <c r="F215">
+        <v>2.53369</v>
+      </c>
+      <c r="G215">
+        <v>7.7684139999999999</v>
+      </c>
+      <c r="H215">
+        <v>26.5154551206181</v>
+      </c>
+    </row>
+    <row r="216" spans="3:8">
+      <c r="C216" t="s">
+        <v>250</v>
+      </c>
+      <c r="D216">
+        <f t="shared" ref="D216:H216" si="1">AVERAGE(D206:D215)</f>
+        <v>204.90863159999998</v>
+      </c>
+      <c r="E216">
+        <f>AVERAGE(E206:E215)</f>
+        <v>10.304414</v>
+      </c>
+      <c r="F216">
+        <f t="shared" si="1"/>
+        <v>2.5361108999999997</v>
+      </c>
+      <c r="G216">
+        <f t="shared" si="1"/>
+        <v>7.7683030999999998</v>
+      </c>
+      <c r="H216">
+        <f t="shared" si="1"/>
+        <v>26.515307729308383</v>
+      </c>
+    </row>
+    <row r="217" spans="3:8">
+      <c r="C217" t="s">
+        <v>251</v>
+      </c>
+      <c r="D217">
+        <f t="shared" ref="D217" si="2">_xlfn.STDEV.S(D206:D215)</f>
+        <v>5.9060142265702368E-3</v>
+      </c>
+      <c r="E217">
+        <f>_xlfn.STDEV.S(E206:E215)</f>
+        <v>1.5310742053284453E-3</v>
+      </c>
+      <c r="F217">
+        <f t="shared" ref="F217:H217" si="3">_xlfn.STDEV.S(F206:F215)</f>
+        <v>1.4163746718686534E-3</v>
+      </c>
+      <c r="G217">
+        <f t="shared" si="3"/>
+        <v>4.6993816378080222E-4</v>
+      </c>
+      <c r="H217">
+        <f t="shared" si="3"/>
+        <v>1.5692796866472723E-3</v>
+      </c>
+    </row>
+    <row r="218" spans="3:8">
+      <c r="C218" t="s">
+        <v>252</v>
+      </c>
+      <c r="D218">
+        <f t="shared" ref="D218:H218" si="4">_xlfn.CONFIDENCE.NORM(0.01,D217,COUNT(D206:D215))</f>
+        <v>4.8107364838944214E-3</v>
+      </c>
+      <c r="E218">
+        <f>_xlfn.CONFIDENCE.NORM(0.01,E217,COUNT(E206:E215))</f>
+        <v>1.2471345744455794E-3</v>
+      </c>
+      <c r="F218">
+        <f t="shared" si="4"/>
+        <v>1.1537062132644844E-3</v>
+      </c>
+      <c r="G218">
+        <f t="shared" si="4"/>
+        <v>3.827875421471052E-4</v>
+      </c>
+      <c r="H218">
+        <f t="shared" si="4"/>
+        <v>1.2782548013556935E-3</v>
+      </c>
+    </row>
+    <row r="220" spans="3:8">
+      <c r="C220" t="s">
+        <v>253</v>
+      </c>
+      <c r="D220" t="s">
+        <v>254</v>
+      </c>
+      <c r="E220" t="s">
+        <v>255</v>
+      </c>
+      <c r="F220" t="s">
+        <v>256</v>
+      </c>
+      <c r="G220" t="s">
+        <v>257</v>
+      </c>
+      <c r="H220" t="s">
+        <v>258</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="C62:G62" xr:uid="{24461DB0-E066-4D80-9F31-EE0FB08E8CE2}">
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C63:G89">
-      <sortCondition ref="D62"/>
+      <sortCondition descending="1" ref="F62"/>
     </sortState>
   </autoFilter>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="C113:C170"/>
     <mergeCell ref="C92:C110"/>
     <mergeCell ref="C28:C59"/>
     <mergeCell ref="I63:I69"/>
+    <mergeCell ref="J174:J183"/>
   </mergeCells>
+  <phoneticPr fontId="3" type="noConversion"/>
   <conditionalFormatting sqref="D63:D81">
     <cfRule type="colorScale" priority="1">
       <colorScale>
@@ -15758,7 +17459,7 @@
       <c r="AA112" s="1"/>
       <c r="AB112" s="1"/>
       <c r="AC112">
-        <f t="shared" ref="AC112:AC143" si="19">SUM(D112:AB112)</f>
+        <f t="shared" ref="AC112:AC115" si="19">SUM(D112:AB112)</f>
         <v>231</v>
       </c>
       <c r="AD112">
@@ -16044,7 +17745,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T20 E20 X20 AB20 E30 E40 E50 E60 E70 E80 E90 E100 E110 T30 T40 T50 T60 T70 T80 T90 T100 T110 X30 X40 X50 X60 X70 X80 X90 X100 X110 AB30 AB40 AB50 AB60 AB70 AB80 AB90 AB100 AB110">
+  <conditionalFormatting sqref="E20 T20 X20 AB20 E30 E40 E50 E60 E70 E80 E90 E100 E110 T30 T40 T50 T60 T70 T80 T90 T100 T110 X30 X40 X50 X60 X70 X80 X90 X100 X110 AB30 AB40 AB50 AB60 AB70 AB80 AB90 AB100 AB110">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -30409,7 +32110,7 @@
       <c r="AA112" s="1"/>
       <c r="AB112" s="1"/>
       <c r="AC112">
-        <f t="shared" ref="AC112:AC143" si="19">SUM(D112:AB112)</f>
+        <f t="shared" ref="AC112:AC115" si="19">SUM(D112:AB112)</f>
         <v>210</v>
       </c>
       <c r="AD112">
@@ -30701,7 +32402,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T20 E20 X20 AB20 E30 E40 E50 E60 E70 E80 E90 E100 E110 T30 T40 T50 T60 T70 T80 T90 T100 T110 X30 X40 X50 X60 X70 X80 X90 X100 X110 AB30 AB40 AB50 AB60 AB70 AB80 AB90 AB100 AB110">
+  <conditionalFormatting sqref="E20 T20 X20 AB20 E30 E40 E50 E60 E70 E80 E90 E100 E110 T30 T40 T50 T60 T70 T80 T90 T100 T110 X30 X40 X50 X60 X70 X80 X90 X100 X110 AB30 AB40 AB50 AB60 AB70 AB80 AB90 AB100 AB110">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -39216,7 +40917,7 @@
       <c r="AA112" s="1"/>
       <c r="AB112" s="1"/>
       <c r="AC112">
-        <f t="shared" ref="AC112:AC143" si="19">SUM(D112:AB112)</f>
+        <f t="shared" ref="AC112:AC115" si="19">SUM(D112:AB112)</f>
         <v>208</v>
       </c>
       <c r="AD112">
@@ -39488,7 +41189,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T20 E20 X20 AB20 E30 E40 E50 E60 E70 E80 E90 E100 E110 T30 T40 T50 T60 T70 T80 T90 T100 T110 X30 X40 X50 X60 X70 X80 X90 X100 X110 AB30 AB40 AB50 AB60 AB70 AB80 AB90 AB100 AB110">
+  <conditionalFormatting sqref="E20 T20 X20 AB20 E30 E40 E50 E60 E70 E80 E90 E100 E110 T30 T40 T50 T60 T70 T80 T90 T100 T110 X30 X40 X50 X60 X70 X80 X90 X100 X110 AB30 AB40 AB50 AB60 AB70 AB80 AB90 AB100 AB110">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -51724,7 +53425,7 @@
       <c r="AA112" s="1"/>
       <c r="AB112" s="1"/>
       <c r="AC112">
-        <f t="shared" ref="AC112:AC143" si="19">SUM(D112:AB112)</f>
+        <f t="shared" ref="AC112:AC115" si="19">SUM(D112:AB112)</f>
         <v>202</v>
       </c>
       <c r="AD112">
@@ -52020,7 +53721,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T20 E20 X20 AB20 E30 E40 E50 E60 E70 E80 E90 E100 E110 T30 T40 T50 T60 T70 T80 T90 T100 T110 X30 X40 X50 X60 X70 X80 X90 X100 X110 AB30 AB40 AB50 AB60 AB70 AB80 AB90 AB100 AB110">
+  <conditionalFormatting sqref="E20 T20 X20 AB20 E30 E40 E50 E60 E70 E80 E90 E100 E110 T30 T40 T50 T60 T70 T80 T90 T100 T110 X30 X40 X50 X60 X70 X80 X90 X100 X110 AB30 AB40 AB50 AB60 AB70 AB80 AB90 AB100 AB110">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -59694,7 +61395,7 @@
       <c r="AA112" s="1"/>
       <c r="AB112" s="1"/>
       <c r="AC112">
-        <f t="shared" ref="AC112:AC143" si="19">SUM(D112:AB112)</f>
+        <f t="shared" ref="AC112:AC115" si="19">SUM(D112:AB112)</f>
         <v>213</v>
       </c>
       <c r="AD112">
@@ -59982,7 +61683,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T20 E20 X20 AB20 E30 E40 E50 E60 E70 E80 E90 E100 E110 T30 T40 T50 T60 T70 T80 T90 T100 T110 X30 X40 X50 X60 X70 X80 X90 X100 X110 AB30 AB40 AB50 AB60 AB70 AB80 AB90 AB100 AB110">
+  <conditionalFormatting sqref="E20 T20 X20 AB20 E30 E40 E50 E60 E70 E80 E90 E100 E110 T30 T40 T50 T60 T70 T80 T90 T100 T110 X30 X40 X50 X60 X70 X80 X90 X100 X110 AB30 AB40 AB50 AB60 AB70 AB80 AB90 AB100 AB110">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>

<commit_message>
Final Solo Trials Complete
Finished strategy testing (result: bank 26 points) added all relevant data to the spreadsheet. Cleaned up code for main game and test enviro. Made minor comment improvements. Plan for further development set out in spreadsheet.
</commit_message>
<xml_diff>
--- a/Flip 7 Data.xlsx
+++ b/Flip 7 Data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b39dc15afb2f4832/Documents/Stuff/Github/Flip-7-Strategy-Finder/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3673" documentId="8_{518FECA9-5F80-4709-BD1F-73FC317A950E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{30C9B9ED-772E-47E0-85E3-322D0AFB8391}"/>
+  <xr:revisionPtr revIDLastSave="3790" documentId="8_{518FECA9-5F80-4709-BD1F-73FC317A950E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DF62B0CA-0697-44E4-9E31-887ABD99303D}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{620B4B94-E82A-42AE-95A9-ED21412A2FCA}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{620B4B94-E82A-42AE-95A9-ED21412A2FCA}"/>
   </bookViews>
   <sheets>
     <sheet name="Master Data" sheetId="1" r:id="rId1"/>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1481" uniqueCount="259">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1522" uniqueCount="267">
   <si>
     <t>Flip 7 Best Strat Test Data</t>
   </si>
@@ -815,9 +815,6 @@
     <t>Test 10</t>
   </si>
   <si>
-    <t>Success vs Bust:</t>
-  </si>
-  <si>
     <t>Mean:</t>
   </si>
   <si>
@@ -830,19 +827,46 @@
     <t>Results: (6 s.f)</t>
   </si>
   <si>
-    <t>204.913 ± 0.00481074</t>
+    <t>Tested with Score 32+</t>
   </si>
   <si>
-    <t>10.3033 ± 0.00124714</t>
+    <t>(Testing other end of spectrum for volatility)</t>
   </si>
   <si>
-    <t>2.53611 ± 0.00115371</t>
+    <t>204.909 ± 0.005</t>
   </si>
   <si>
-    <t>7.76830 ± 0.000382788</t>
+    <t>10.3044 ± 0.0012</t>
   </si>
   <si>
-    <t>26.5153 ± 0.00127826</t>
+    <t>2.53611 ± 0.00115</t>
+  </si>
+  <si>
+    <t>7.76830 ± 0.00038</t>
+  </si>
+  <si>
+    <t>26.5153 ± 0.00128</t>
+  </si>
+  <si>
+    <t>204.781 ± 0.005</t>
+  </si>
+  <si>
+    <t>4.47366 ± 0.00256</t>
+  </si>
+  <si>
+    <t>5.92550 ± 0.00027</t>
+  </si>
+  <si>
+    <t>34.6549 ± 0.0019</t>
+  </si>
+  <si>
+    <t>10.3991 ± 0.0025</t>
+  </si>
+  <si>
+    <t>Final Conclusion and Takeaways</t>
+  </si>
+  <si>
+    <t>I can now say for certain that the best and most efficient strategy according to my method of testing is to always bank as soon as you've flipped ~25-26 points worth of cards. In practice this strategy probably won't always prevail since other players can discard or swap your cards to force you to bust sooner and bank a score lower than otherwise. In a similar vain, other players may gamble harder than you and get lucky. This strategy is simply the most consistent gameplan and has the quickest time to finish in solo play. If I were to develop this further, I would need to develop player AI's to play against and around to see how that impacts gameplay and if things like the discard have optimal use cases that can be exploited to give you an even further edge. However for right now I'm content with wha I've managed so far and what I've learned through using excel so extensively and working with these large volumes of data.</t>
   </si>
 </sst>
 </file>
@@ -930,7 +954,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -946,13 +970,22 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -3588,6 +3621,334 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-GB"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Master Data'!$E$173</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Average Rounds to 200</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Master Data'!$E$174:$E$188</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>10.695829</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>10.532031</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>10.372769999999999</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>10.306252000000001</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>10.226029</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>10.118207999999999</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>10.109500000000001</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>10.168869000000001</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>10.235564</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>10.247678000000001</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>10.229124000000001</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>10.260602</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>10.400808</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>10.639106</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>10.911483</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-367B-4D96-BF83-DC06D8BB7E1E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1188395936"/>
+        <c:axId val="1188402656"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1188395936"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1188402656"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1188402656"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1188395936"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -3709,6 +4070,46 @@
 </file>
 
 <file path=xl/charts/colors4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors5.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -5799,6 +6200,522 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style5.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
@@ -5911,16 +6828,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>668365</xdr:colOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>36815</xdr:colOff>
       <xdr:row>188</xdr:row>
-      <xdr:rowOff>129798</xdr:rowOff>
+      <xdr:rowOff>57324</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>857251</xdr:colOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>28990</xdr:colOff>
       <xdr:row>202</xdr:row>
-      <xdr:rowOff>160795</xdr:rowOff>
+      <xdr:rowOff>88321</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -5940,6 +6857,42 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>668656</xdr:colOff>
+      <xdr:row>188</xdr:row>
+      <xdr:rowOff>42903</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>311592</xdr:colOff>
+      <xdr:row>202</xdr:row>
+      <xdr:rowOff>114961</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{82572512-534B-6C92-7762-805D3DFC7A88}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -6521,7 +7474,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24461DB0-E066-4D80-9F31-EE0FB08E8CE2}">
-  <dimension ref="C2:CS220"/>
+  <dimension ref="C2:CS274"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="3" max="3" width="28.28515625" bestFit="1" customWidth="1"/>
@@ -6676,19 +7629,19 @@
         <v>16</v>
       </c>
       <c r="D11" s="2">
-        <f>'Flip7 or Bust'!T13</f>
+        <f>'Flip7 or Bust'!AH13</f>
         <v>0</v>
       </c>
       <c r="E11" s="2">
-        <f>'Flip7 or Bust'!U13</f>
+        <f>'Flip7 or Bust'!AI13</f>
         <v>0</v>
       </c>
       <c r="F11" s="2">
-        <f>'Flip7 or Bust'!V13</f>
+        <f>'Flip7 or Bust'!AJ13</f>
         <v>0</v>
       </c>
       <c r="G11" s="2" t="e">
-        <f>'Flip7 or Bust'!W13</f>
+        <f>'Flip7 or Bust'!AK13</f>
         <v>#DIV/0!</v>
       </c>
       <c r="H11" s="3"/>
@@ -7522,18 +8475,18 @@
       </c>
     </row>
     <row r="28" spans="3:97" ht="15" customHeight="1">
-      <c r="C28" s="9" t="s">
+      <c r="C28" s="8" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="29" spans="3:97">
-      <c r="C29" s="9"/>
+      <c r="C29" s="8"/>
       <c r="K29" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="30" spans="3:97">
-      <c r="C30" s="9"/>
+      <c r="C30" s="8"/>
       <c r="K30" t="s">
         <v>98</v>
       </c>
@@ -7545,7 +8498,7 @@
       </c>
     </row>
     <row r="31" spans="3:97">
-      <c r="C31" s="9"/>
+      <c r="C31" s="8"/>
       <c r="K31">
         <v>-8.79120879120876E-2</v>
       </c>
@@ -7557,7 +8510,7 @@
       </c>
     </row>
     <row r="32" spans="3:97">
-      <c r="C32" s="9"/>
+      <c r="C32" s="8"/>
       <c r="K32">
         <v>-0.22222222222222099</v>
       </c>
@@ -7569,7 +8522,7 @@
       </c>
     </row>
     <row r="33" spans="3:15">
-      <c r="C33" s="9"/>
+      <c r="C33" s="8"/>
       <c r="K33">
         <v>-0.46067415730336903</v>
       </c>
@@ -7581,7 +8534,7 @@
       </c>
     </row>
     <row r="34" spans="3:15">
-      <c r="C34" s="9"/>
+      <c r="C34" s="8"/>
       <c r="K34">
         <v>0.5</v>
       </c>
@@ -7593,7 +8546,7 @@
       </c>
     </row>
     <row r="35" spans="3:15">
-      <c r="C35" s="9"/>
+      <c r="C35" s="8"/>
       <c r="K35">
         <v>-0.42528735632183801</v>
       </c>
@@ -7605,7 +8558,7 @@
       </c>
     </row>
     <row r="36" spans="3:15">
-      <c r="C36" s="9"/>
+      <c r="C36" s="8"/>
       <c r="K36">
         <v>-0.32558139534884101</v>
       </c>
@@ -7617,7 +8570,7 @@
       </c>
     </row>
     <row r="37" spans="3:15">
-      <c r="C37" s="9"/>
+      <c r="C37" s="8"/>
       <c r="K37">
         <v>0.66666666666666696</v>
       </c>
@@ -7629,7 +8582,7 @@
       </c>
     </row>
     <row r="38" spans="3:15">
-      <c r="C38" s="9"/>
+      <c r="C38" s="8"/>
       <c r="K38">
         <v>1.5180722891566201</v>
       </c>
@@ -7641,7 +8594,7 @@
       </c>
     </row>
     <row r="39" spans="3:15">
-      <c r="C39" s="9"/>
+      <c r="C39" s="8"/>
       <c r="K39">
         <v>1.17073170731707</v>
       </c>
@@ -7653,7 +8606,7 @@
       </c>
     </row>
     <row r="40" spans="3:15">
-      <c r="C40" s="9"/>
+      <c r="C40" s="8"/>
       <c r="K40">
         <v>2.9012345679012301</v>
       </c>
@@ -7665,7 +8618,7 @@
       </c>
     </row>
     <row r="41" spans="3:15">
-      <c r="C41" s="9"/>
+      <c r="C41" s="8"/>
       <c r="K41">
         <v>1.75</v>
       </c>
@@ -7677,7 +8630,7 @@
       </c>
     </row>
     <row r="42" spans="3:15">
-      <c r="C42" s="9"/>
+      <c r="C42" s="8"/>
       <c r="K42">
         <v>-0.82051282051281904</v>
       </c>
@@ -7689,7 +8642,7 @@
       </c>
     </row>
     <row r="43" spans="3:15">
-      <c r="C43" s="9"/>
+      <c r="C43" s="8"/>
       <c r="K43">
         <v>12.012987012987001</v>
       </c>
@@ -7701,7 +8654,7 @@
       </c>
     </row>
     <row r="44" spans="3:15">
-      <c r="C44" s="9"/>
+      <c r="C44" s="8"/>
       <c r="K44">
         <v>11.3157894736842</v>
       </c>
@@ -7713,7 +8666,7 @@
       </c>
     </row>
     <row r="45" spans="3:15">
-      <c r="C45" s="9"/>
+      <c r="C45" s="8"/>
       <c r="K45">
         <v>12.6666666666666</v>
       </c>
@@ -7725,7 +8678,7 @@
       </c>
     </row>
     <row r="46" spans="3:15">
-      <c r="C46" s="9"/>
+      <c r="C46" s="8"/>
       <c r="K46">
         <v>12.270270270270199</v>
       </c>
@@ -7737,7 +8690,7 @@
       </c>
     </row>
     <row r="47" spans="3:15">
-      <c r="C47" s="9"/>
+      <c r="C47" s="8"/>
       <c r="K47">
         <v>12.8630136986301</v>
       </c>
@@ -7749,7 +8702,7 @@
       </c>
     </row>
     <row r="48" spans="3:15">
-      <c r="C48" s="9"/>
+      <c r="C48" s="8"/>
       <c r="K48">
         <v>2.77464788732394</v>
       </c>
@@ -7761,7 +8714,7 @@
       </c>
     </row>
     <row r="49" spans="3:15">
-      <c r="C49" s="9"/>
+      <c r="C49" s="8"/>
       <c r="K49">
         <v>3.5714285714285698</v>
       </c>
@@ -7773,7 +8726,7 @@
       </c>
     </row>
     <row r="50" spans="3:15">
-      <c r="C50" s="9"/>
+      <c r="C50" s="8"/>
       <c r="K50">
         <v>3.3623188405797002</v>
       </c>
@@ -7785,7 +8738,7 @@
       </c>
     </row>
     <row r="51" spans="3:15">
-      <c r="C51" s="9"/>
+      <c r="C51" s="8"/>
       <c r="K51">
         <v>2.70588235294117</v>
       </c>
@@ -7797,7 +8750,7 @@
       </c>
     </row>
     <row r="52" spans="3:15">
-      <c r="C52" s="9"/>
+      <c r="C52" s="8"/>
       <c r="K52">
         <v>2.2089552238805998</v>
       </c>
@@ -7809,7 +8762,7 @@
       </c>
     </row>
     <row r="53" spans="3:15">
-      <c r="C53" s="9"/>
+      <c r="C53" s="8"/>
       <c r="K53">
         <v>0.51515151515151503</v>
       </c>
@@ -7821,7 +8774,7 @@
       </c>
     </row>
     <row r="54" spans="3:15">
-      <c r="C54" s="9"/>
+      <c r="C54" s="8"/>
       <c r="K54">
         <v>5.48484848484848</v>
       </c>
@@ -7833,7 +8786,7 @@
       </c>
     </row>
     <row r="55" spans="3:15">
-      <c r="C55" s="9"/>
+      <c r="C55" s="8"/>
       <c r="K55">
         <v>6.2307692307692299</v>
       </c>
@@ -7845,7 +8798,7 @@
       </c>
     </row>
     <row r="56" spans="3:15">
-      <c r="C56" s="9"/>
+      <c r="C56" s="8"/>
       <c r="K56">
         <v>5.5625</v>
       </c>
@@ -7857,7 +8810,7 @@
       </c>
     </row>
     <row r="57" spans="3:15">
-      <c r="C57" s="9"/>
+      <c r="C57" s="8"/>
       <c r="K57">
         <v>5.4920634920634903</v>
       </c>
@@ -7869,7 +8822,7 @@
       </c>
     </row>
     <row r="58" spans="3:15">
-      <c r="C58" s="9"/>
+      <c r="C58" s="8"/>
       <c r="K58">
         <v>1.38709677419355</v>
       </c>
@@ -7881,7 +8834,7 @@
       </c>
     </row>
     <row r="59" spans="3:15">
-      <c r="C59" s="9"/>
+      <c r="C59" s="8"/>
       <c r="K59">
         <v>-0.66666666666666596</v>
       </c>
@@ -7964,7 +8917,7 @@
         <v>24.296027417027421</v>
       </c>
       <c r="H63" s="4"/>
-      <c r="I63" s="10" t="s">
+      <c r="I63" s="12" t="s">
         <v>207</v>
       </c>
       <c r="K63">
@@ -7998,7 +8951,7 @@
         <v>24.679059523809524</v>
       </c>
       <c r="H64" s="4"/>
-      <c r="I64" s="10"/>
+      <c r="I64" s="12"/>
       <c r="K64">
         <v>1.4814814814814801</v>
       </c>
@@ -8030,7 +8983,7 @@
         <v>25.835992063492068</v>
       </c>
       <c r="H65" s="4"/>
-      <c r="I65" s="10"/>
+      <c r="I65" s="12"/>
       <c r="K65">
         <v>6.2452830188679203</v>
       </c>
@@ -8062,7 +9015,7 @@
         <v>26.310999999999993</v>
       </c>
       <c r="H66" s="4"/>
-      <c r="I66" s="10"/>
+      <c r="I66" s="12"/>
       <c r="K66">
         <v>6.1538461538461497</v>
       </c>
@@ -8094,7 +9047,7 @@
         <v>26.516269841269835</v>
       </c>
       <c r="H67" s="4"/>
-      <c r="I67" s="10"/>
+      <c r="I67" s="12"/>
       <c r="K67">
         <v>-1</v>
       </c>
@@ -8126,7 +9079,7 @@
         <v>27.740297619047613</v>
       </c>
       <c r="H68" s="4"/>
-      <c r="I68" s="10"/>
+      <c r="I68" s="12"/>
       <c r="K68">
         <v>0.63265306122448794</v>
       </c>
@@ -8158,7 +9111,7 @@
         <v>28.177678571428572</v>
       </c>
       <c r="H69" s="4"/>
-      <c r="I69" s="10"/>
+      <c r="I69" s="12"/>
       <c r="K69">
         <v>-18.75</v>
       </c>
@@ -8681,7 +9634,7 @@
       </c>
     </row>
     <row r="92" spans="3:15" ht="15" customHeight="1">
-      <c r="C92" s="8" t="s">
+      <c r="C92" s="11" t="s">
         <v>206</v>
       </c>
       <c r="K92">
@@ -8695,7 +9648,7 @@
       </c>
     </row>
     <row r="93" spans="3:15">
-      <c r="C93" s="8"/>
+      <c r="C93" s="11"/>
       <c r="K93">
         <v>-20.105263157894701</v>
       </c>
@@ -8707,7 +9660,7 @@
       </c>
     </row>
     <row r="94" spans="3:15">
-      <c r="C94" s="8"/>
+      <c r="C94" s="11"/>
       <c r="K94">
         <v>-14.529411764705801</v>
       </c>
@@ -8719,7 +9672,7 @@
       </c>
     </row>
     <row r="95" spans="3:15">
-      <c r="C95" s="8"/>
+      <c r="C95" s="11"/>
       <c r="K95">
         <v>-4.3333333333333304</v>
       </c>
@@ -8731,7 +9684,7 @@
       </c>
     </row>
     <row r="96" spans="3:15">
-      <c r="C96" s="8"/>
+      <c r="C96" s="11"/>
       <c r="K96">
         <v>0.57142857142857295</v>
       </c>
@@ -8743,7 +9696,7 @@
       </c>
     </row>
     <row r="97" spans="3:15">
-      <c r="C97" s="8"/>
+      <c r="C97" s="11"/>
       <c r="K97">
         <v>2.9230769230769198</v>
       </c>
@@ -8755,7 +9708,7 @@
       </c>
     </row>
     <row r="98" spans="3:15">
-      <c r="C98" s="8"/>
+      <c r="C98" s="11"/>
       <c r="K98">
         <v>-3.6666666666666701</v>
       </c>
@@ -8767,7 +9720,7 @@
       </c>
     </row>
     <row r="99" spans="3:15">
-      <c r="C99" s="8"/>
+      <c r="C99" s="11"/>
       <c r="K99">
         <v>0</v>
       </c>
@@ -8779,7 +9732,7 @@
       </c>
     </row>
     <row r="100" spans="3:15">
-      <c r="C100" s="8"/>
+      <c r="C100" s="11"/>
       <c r="K100">
         <v>-0.22222222222222099</v>
       </c>
@@ -8791,7 +9744,7 @@
       </c>
     </row>
     <row r="101" spans="3:15">
-      <c r="C101" s="8"/>
+      <c r="C101" s="11"/>
       <c r="L101">
         <v>6.3999999999999897</v>
       </c>
@@ -8800,7 +9753,7 @@
       </c>
     </row>
     <row r="102" spans="3:15">
-      <c r="C102" s="8"/>
+      <c r="C102" s="11"/>
       <c r="L102">
         <v>7.3999999999999897</v>
       </c>
@@ -8809,7 +9762,7 @@
       </c>
     </row>
     <row r="103" spans="3:15">
-      <c r="C103" s="8"/>
+      <c r="C103" s="11"/>
       <c r="L103">
         <v>16.399999999999999</v>
       </c>
@@ -8818,7 +9771,7 @@
       </c>
     </row>
     <row r="104" spans="3:15">
-      <c r="C104" s="8"/>
+      <c r="C104" s="11"/>
       <c r="L104">
         <v>-9.9626373626373592</v>
       </c>
@@ -8827,7 +9780,7 @@
       </c>
     </row>
     <row r="105" spans="3:15">
-      <c r="C105" s="8"/>
+      <c r="C105" s="11"/>
       <c r="L105">
         <v>-7.1123595505617896</v>
       </c>
@@ -8836,7 +9789,7 @@
       </c>
     </row>
     <row r="106" spans="3:15">
-      <c r="C106" s="8"/>
+      <c r="C106" s="11"/>
       <c r="L106">
         <v>-6.7272727272727204</v>
       </c>
@@ -8845,7 +9798,7 @@
       </c>
     </row>
     <row r="107" spans="3:15">
-      <c r="C107" s="8"/>
+      <c r="C107" s="11"/>
       <c r="L107">
         <v>-7.0344827586206904</v>
       </c>
@@ -8854,7 +9807,7 @@
       </c>
     </row>
     <row r="108" spans="3:15">
-      <c r="C108" s="8"/>
+      <c r="C108" s="11"/>
       <c r="L108">
         <v>-6.53488372093023</v>
       </c>
@@ -8863,7 +9816,7 @@
       </c>
     </row>
     <row r="109" spans="3:15">
-      <c r="C109" s="8"/>
+      <c r="C109" s="11"/>
       <c r="L109">
         <v>-6.3523809523809502</v>
       </c>
@@ -8872,7 +9825,7 @@
       </c>
     </row>
     <row r="110" spans="3:15">
-      <c r="C110" s="8"/>
+      <c r="C110" s="11"/>
       <c r="L110">
         <v>5.9523809523809499</v>
       </c>
@@ -8889,190 +9842,190 @@
       </c>
     </row>
     <row r="113" spans="3:3" ht="15" customHeight="1">
-      <c r="C113" s="8" t="s">
+      <c r="C113" s="11" t="s">
         <v>219</v>
       </c>
     </row>
     <row r="114" spans="3:3">
-      <c r="C114" s="8"/>
+      <c r="C114" s="11"/>
     </row>
     <row r="115" spans="3:3">
-      <c r="C115" s="8"/>
+      <c r="C115" s="11"/>
     </row>
     <row r="116" spans="3:3">
-      <c r="C116" s="8"/>
+      <c r="C116" s="11"/>
     </row>
     <row r="117" spans="3:3">
-      <c r="C117" s="8"/>
+      <c r="C117" s="11"/>
     </row>
     <row r="118" spans="3:3">
-      <c r="C118" s="8"/>
+      <c r="C118" s="11"/>
     </row>
     <row r="119" spans="3:3">
-      <c r="C119" s="8"/>
+      <c r="C119" s="11"/>
     </row>
     <row r="120" spans="3:3">
-      <c r="C120" s="8"/>
+      <c r="C120" s="11"/>
     </row>
     <row r="121" spans="3:3">
-      <c r="C121" s="8"/>
+      <c r="C121" s="11"/>
     </row>
     <row r="122" spans="3:3">
-      <c r="C122" s="8"/>
+      <c r="C122" s="11"/>
     </row>
     <row r="123" spans="3:3">
-      <c r="C123" s="8"/>
+      <c r="C123" s="11"/>
     </row>
     <row r="124" spans="3:3">
-      <c r="C124" s="8"/>
+      <c r="C124" s="11"/>
     </row>
     <row r="125" spans="3:3">
-      <c r="C125" s="8"/>
+      <c r="C125" s="11"/>
     </row>
     <row r="126" spans="3:3">
-      <c r="C126" s="8"/>
+      <c r="C126" s="11"/>
     </row>
     <row r="127" spans="3:3">
-      <c r="C127" s="8"/>
+      <c r="C127" s="11"/>
     </row>
     <row r="128" spans="3:3">
-      <c r="C128" s="8"/>
+      <c r="C128" s="11"/>
     </row>
     <row r="129" spans="3:3">
-      <c r="C129" s="8"/>
+      <c r="C129" s="11"/>
     </row>
     <row r="130" spans="3:3">
-      <c r="C130" s="8"/>
+      <c r="C130" s="11"/>
     </row>
     <row r="131" spans="3:3">
-      <c r="C131" s="8"/>
+      <c r="C131" s="11"/>
     </row>
     <row r="132" spans="3:3">
-      <c r="C132" s="8"/>
+      <c r="C132" s="11"/>
     </row>
     <row r="133" spans="3:3">
-      <c r="C133" s="8"/>
+      <c r="C133" s="11"/>
     </row>
     <row r="134" spans="3:3">
-      <c r="C134" s="8"/>
+      <c r="C134" s="11"/>
     </row>
     <row r="135" spans="3:3">
-      <c r="C135" s="8"/>
+      <c r="C135" s="11"/>
     </row>
     <row r="136" spans="3:3">
-      <c r="C136" s="8"/>
+      <c r="C136" s="11"/>
     </row>
     <row r="137" spans="3:3">
-      <c r="C137" s="8"/>
+      <c r="C137" s="11"/>
     </row>
     <row r="138" spans="3:3">
-      <c r="C138" s="8"/>
+      <c r="C138" s="11"/>
     </row>
     <row r="139" spans="3:3">
-      <c r="C139" s="8"/>
+      <c r="C139" s="11"/>
     </row>
     <row r="140" spans="3:3">
-      <c r="C140" s="8"/>
+      <c r="C140" s="11"/>
     </row>
     <row r="141" spans="3:3">
-      <c r="C141" s="8"/>
+      <c r="C141" s="11"/>
     </row>
     <row r="142" spans="3:3">
-      <c r="C142" s="8"/>
+      <c r="C142" s="11"/>
     </row>
     <row r="143" spans="3:3">
-      <c r="C143" s="8"/>
+      <c r="C143" s="11"/>
     </row>
     <row r="144" spans="3:3">
-      <c r="C144" s="8"/>
+      <c r="C144" s="11"/>
     </row>
     <row r="145" spans="3:3">
-      <c r="C145" s="8"/>
+      <c r="C145" s="11"/>
     </row>
     <row r="146" spans="3:3">
-      <c r="C146" s="8"/>
+      <c r="C146" s="11"/>
     </row>
     <row r="147" spans="3:3">
-      <c r="C147" s="8"/>
+      <c r="C147" s="11"/>
     </row>
     <row r="148" spans="3:3">
-      <c r="C148" s="8"/>
+      <c r="C148" s="11"/>
     </row>
     <row r="149" spans="3:3">
-      <c r="C149" s="8"/>
+      <c r="C149" s="11"/>
     </row>
     <row r="150" spans="3:3">
-      <c r="C150" s="8"/>
+      <c r="C150" s="11"/>
     </row>
     <row r="151" spans="3:3">
-      <c r="C151" s="8"/>
+      <c r="C151" s="11"/>
     </row>
     <row r="152" spans="3:3">
-      <c r="C152" s="8"/>
+      <c r="C152" s="11"/>
     </row>
     <row r="153" spans="3:3">
-      <c r="C153" s="8"/>
+      <c r="C153" s="11"/>
     </row>
     <row r="154" spans="3:3">
-      <c r="C154" s="8"/>
+      <c r="C154" s="11"/>
     </row>
     <row r="155" spans="3:3">
-      <c r="C155" s="8"/>
+      <c r="C155" s="11"/>
     </row>
     <row r="156" spans="3:3">
-      <c r="C156" s="8"/>
+      <c r="C156" s="11"/>
     </row>
     <row r="157" spans="3:3">
-      <c r="C157" s="8"/>
+      <c r="C157" s="11"/>
     </row>
     <row r="158" spans="3:3">
-      <c r="C158" s="8"/>
+      <c r="C158" s="11"/>
     </row>
     <row r="159" spans="3:3">
-      <c r="C159" s="8"/>
+      <c r="C159" s="11"/>
     </row>
     <row r="160" spans="3:3">
-      <c r="C160" s="8"/>
-    </row>
-    <row r="161" spans="3:10">
-      <c r="C161" s="8"/>
-    </row>
-    <row r="162" spans="3:10">
-      <c r="C162" s="8"/>
-    </row>
-    <row r="163" spans="3:10">
-      <c r="C163" s="8"/>
-    </row>
-    <row r="164" spans="3:10">
-      <c r="C164" s="8"/>
-    </row>
-    <row r="165" spans="3:10">
-      <c r="C165" s="8"/>
-    </row>
-    <row r="166" spans="3:10">
-      <c r="C166" s="8"/>
-    </row>
-    <row r="167" spans="3:10">
-      <c r="C167" s="8"/>
-    </row>
-    <row r="168" spans="3:10">
-      <c r="C168" s="8"/>
-    </row>
-    <row r="169" spans="3:10">
-      <c r="C169" s="8"/>
-    </row>
-    <row r="170" spans="3:10">
-      <c r="C170" s="8"/>
-    </row>
-    <row r="171" spans="3:10">
+      <c r="C160" s="11"/>
+    </row>
+    <row r="161" spans="3:9">
+      <c r="C161" s="11"/>
+    </row>
+    <row r="162" spans="3:9">
+      <c r="C162" s="11"/>
+    </row>
+    <row r="163" spans="3:9">
+      <c r="C163" s="11"/>
+    </row>
+    <row r="164" spans="3:9">
+      <c r="C164" s="11"/>
+    </row>
+    <row r="165" spans="3:9">
+      <c r="C165" s="11"/>
+    </row>
+    <row r="166" spans="3:9">
+      <c r="C166" s="11"/>
+    </row>
+    <row r="167" spans="3:9">
+      <c r="C167" s="11"/>
+    </row>
+    <row r="168" spans="3:9">
+      <c r="C168" s="11"/>
+    </row>
+    <row r="169" spans="3:9">
+      <c r="C169" s="11"/>
+    </row>
+    <row r="170" spans="3:9">
+      <c r="C170" s="11"/>
+    </row>
+    <row r="171" spans="3:9">
       <c r="C171" s="7"/>
     </row>
-    <row r="172" spans="3:10">
+    <row r="172" spans="3:9">
       <c r="C172" t="s">
         <v>220</v>
       </c>
     </row>
-    <row r="173" spans="3:10">
+    <row r="173" spans="3:9">
       <c r="D173" t="s">
         <v>228</v>
       </c>
@@ -9088,11 +10041,8 @@
       <c r="H173" t="s">
         <v>229</v>
       </c>
-      <c r="I173" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="174" spans="3:10" ht="15" customHeight="1">
+    </row>
+    <row r="174" spans="3:9" ht="15" customHeight="1">
       <c r="C174" s="7" t="s">
         <v>221</v>
       </c>
@@ -9111,15 +10061,11 @@
       <c r="H174">
         <v>23.6955327936281</v>
       </c>
-      <c r="I174">
-        <f>G174/F174</f>
-        <v>4.3469520486312456</v>
-      </c>
-      <c r="J174" s="9" t="s">
+      <c r="I174" s="8" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="175" spans="3:10">
+    <row r="175" spans="3:9">
       <c r="C175" s="7" t="s">
         <v>222</v>
       </c>
@@ -9138,13 +10084,9 @@
       <c r="H175">
         <v>24.641126278171399</v>
       </c>
-      <c r="I175">
-        <f t="shared" ref="I175:I188" si="0">G175/F175</f>
-        <v>3.8609209322676135</v>
-      </c>
-      <c r="J175" s="9"/>
-    </row>
-    <row r="176" spans="3:10">
+      <c r="I175" s="8"/>
+    </row>
+    <row r="176" spans="3:9">
       <c r="C176" s="7" t="s">
         <v>223</v>
       </c>
@@ -9163,13 +10105,9 @@
       <c r="H176">
         <v>25.710231051580699</v>
       </c>
-      <c r="I176">
-        <f t="shared" si="0"/>
-        <v>3.3873220373393789</v>
-      </c>
-      <c r="J176" s="9"/>
-    </row>
-    <row r="177" spans="3:10">
+      <c r="I176" s="8"/>
+    </row>
+    <row r="177" spans="3:9">
       <c r="C177" s="7" t="s">
         <v>224</v>
       </c>
@@ -9188,13 +10126,9 @@
       <c r="H177">
         <v>26.514071702364198</v>
       </c>
-      <c r="I177">
-        <f t="shared" si="0"/>
-        <v>3.0610826110239184</v>
-      </c>
-      <c r="J177" s="9"/>
-    </row>
-    <row r="178" spans="3:10">
+      <c r="I177" s="8"/>
+    </row>
+    <row r="178" spans="3:9">
       <c r="C178" s="7" t="s">
         <v>225</v>
       </c>
@@ -9213,13 +10147,9 @@
       <c r="H178">
         <v>27.661426526549299</v>
       </c>
-      <c r="I178">
-        <f t="shared" si="0"/>
-        <v>2.6918991456595576</v>
-      </c>
-      <c r="J178" s="9"/>
-    </row>
-    <row r="179" spans="3:10">
+      <c r="I178" s="8"/>
+    </row>
+    <row r="179" spans="3:9">
       <c r="C179" s="7" t="s">
         <v>226</v>
       </c>
@@ -9238,13 +10168,9 @@
       <c r="H179">
         <v>28.770401677324799</v>
       </c>
-      <c r="I179">
-        <f t="shared" si="0"/>
-        <v>2.4177246487936199</v>
-      </c>
-      <c r="J179" s="9"/>
-    </row>
-    <row r="180" spans="3:10">
+      <c r="I179" s="8"/>
+    </row>
+    <row r="180" spans="3:9">
       <c r="C180" s="7" t="s">
         <v>227</v>
       </c>
@@ -9263,13 +10189,9 @@
       <c r="H180">
         <v>29.576063808268401</v>
       </c>
-      <c r="I180">
-        <f t="shared" si="0"/>
-        <v>2.1971297146950324</v>
-      </c>
-      <c r="J180" s="9"/>
-    </row>
-    <row r="181" spans="3:10">
+      <c r="I180" s="8"/>
+    </row>
+    <row r="181" spans="3:9">
       <c r="C181" s="7" t="s">
         <v>231</v>
       </c>
@@ -9288,13 +10210,9 @@
       <c r="H181">
         <v>29.997730984461601</v>
       </c>
-      <c r="I181">
-        <f t="shared" si="0"/>
-        <v>2.0689902442336856</v>
-      </c>
-      <c r="J181" s="9"/>
-    </row>
-    <row r="182" spans="3:10">
+      <c r="I181" s="8"/>
+    </row>
+    <row r="182" spans="3:9">
       <c r="C182" s="7" t="s">
         <v>232</v>
       </c>
@@ -9313,13 +10231,9 @@
       <c r="H182">
         <v>30.680995797563401</v>
       </c>
-      <c r="I182">
-        <f t="shared" si="0"/>
-        <v>1.9100735879670894</v>
-      </c>
-      <c r="J182" s="9"/>
-    </row>
-    <row r="183" spans="3:10">
+      <c r="I182" s="8"/>
+    </row>
+    <row r="183" spans="3:9">
       <c r="C183" s="7" t="s">
         <v>233</v>
       </c>
@@ -9338,13 +10252,9 @@
       <c r="H183">
         <v>31.856338171378201</v>
       </c>
-      <c r="I183">
-        <f t="shared" si="0"/>
-        <v>1.7206114028208381</v>
-      </c>
-      <c r="J183" s="9"/>
-    </row>
-    <row r="184" spans="3:10">
+      <c r="I183" s="8"/>
+    </row>
+    <row r="184" spans="3:9">
       <c r="C184" s="7" t="s">
         <v>234</v>
       </c>
@@ -9363,12 +10273,8 @@
       <c r="H184">
         <v>33.190480828526397</v>
       </c>
-      <c r="I184">
-        <f t="shared" si="0"/>
-        <v>1.5461333914787583</v>
-      </c>
-    </row>
-    <row r="185" spans="3:10">
+    </row>
+    <row r="185" spans="3:9">
       <c r="C185" s="7" t="s">
         <v>235</v>
       </c>
@@ -9387,12 +10293,8 @@
       <c r="H185">
         <v>34.217799095202501</v>
       </c>
-      <c r="I185">
-        <f t="shared" si="0"/>
-        <v>1.4119030067566931</v>
-      </c>
-    </row>
-    <row r="186" spans="3:10">
+    </row>
+    <row r="186" spans="3:9">
       <c r="C186" s="7" t="s">
         <v>236</v>
       </c>
@@ -9411,12 +10313,8 @@
       <c r="H186">
         <v>34.654331254727502</v>
       </c>
-      <c r="I186">
-        <f t="shared" si="0"/>
-        <v>1.3241275981001732</v>
-      </c>
-    </row>
-    <row r="187" spans="3:10">
+    </row>
+    <row r="187" spans="3:9">
       <c r="C187" s="7" t="s">
         <v>237</v>
       </c>
@@ -9435,12 +10333,8 @@
       <c r="H187">
         <v>34.957205602348502</v>
       </c>
-      <c r="I187">
-        <f t="shared" si="0"/>
-        <v>1.2357582421092537</v>
-      </c>
-    </row>
-    <row r="188" spans="3:10">
+    </row>
+    <row r="188" spans="3:9">
       <c r="C188" s="7" t="s">
         <v>238</v>
       </c>
@@ -9459,21 +10353,17 @@
       <c r="H188">
         <v>35.557773966639303</v>
       </c>
-      <c r="I188">
-        <f t="shared" si="0"/>
-        <v>1.1324914101200814</v>
-      </c>
-    </row>
-    <row r="189" spans="3:10">
+    </row>
+    <row r="189" spans="3:9">
       <c r="C189" s="7"/>
     </row>
-    <row r="190" spans="3:10">
+    <row r="190" spans="3:9">
       <c r="C190" s="7"/>
     </row>
-    <row r="191" spans="3:10">
+    <row r="191" spans="3:9">
       <c r="C191" s="7"/>
     </row>
-    <row r="192" spans="3:10">
+    <row r="192" spans="3:9">
       <c r="C192" s="7"/>
     </row>
     <row r="193" spans="3:8">
@@ -9733,10 +10623,10 @@
     </row>
     <row r="216" spans="3:8">
       <c r="C216" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D216">
-        <f t="shared" ref="D216:H216" si="1">AVERAGE(D206:D215)</f>
+        <f t="shared" ref="D216:H216" si="0">AVERAGE(D206:D215)</f>
         <v>204.90863159999998</v>
       </c>
       <c r="E216">
@@ -9744,24 +10634,24 @@
         <v>10.304414</v>
       </c>
       <c r="F216">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>2.5361108999999997</v>
       </c>
       <c r="G216">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>7.7683030999999998</v>
       </c>
       <c r="H216">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>26.515307729308383</v>
       </c>
     </row>
     <row r="217" spans="3:8">
       <c r="C217" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="D217">
-        <f t="shared" ref="D217" si="2">_xlfn.STDEV.S(D206:D215)</f>
+        <f t="shared" ref="D217" si="1">_xlfn.STDEV.S(D206:D215)</f>
         <v>5.9060142265702368E-3</v>
       </c>
       <c r="E217">
@@ -9769,24 +10659,24 @@
         <v>1.5310742053284453E-3</v>
       </c>
       <c r="F217">
-        <f t="shared" ref="F217:H217" si="3">_xlfn.STDEV.S(F206:F215)</f>
+        <f t="shared" ref="F217:H217" si="2">_xlfn.STDEV.S(F206:F215)</f>
         <v>1.4163746718686534E-3</v>
       </c>
       <c r="G217">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>4.6993816378080222E-4</v>
       </c>
       <c r="H217">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>1.5692796866472723E-3</v>
       </c>
     </row>
     <row r="218" spans="3:8">
       <c r="C218" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D218">
-        <f t="shared" ref="D218:H218" si="4">_xlfn.CONFIDENCE.NORM(0.01,D217,COUNT(D206:D215))</f>
+        <f t="shared" ref="D218:H218" si="3">_xlfn.CONFIDENCE.NORM(0.01,D217,COUNT(D206:D215))</f>
         <v>4.8107364838944214E-3</v>
       </c>
       <c r="E218">
@@ -9794,37 +10684,459 @@
         <v>1.2471345744455794E-3</v>
       </c>
       <c r="F218">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>1.1537062132644844E-3</v>
       </c>
       <c r="G218">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>3.827875421471052E-4</v>
       </c>
       <c r="H218">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>1.2782548013556935E-3</v>
       </c>
     </row>
     <row r="220" spans="3:8">
       <c r="C220" t="s">
+        <v>252</v>
+      </c>
+      <c r="D220" t="s">
+        <v>255</v>
+      </c>
+      <c r="E220" t="s">
+        <v>256</v>
+      </c>
+      <c r="F220" t="s">
+        <v>257</v>
+      </c>
+      <c r="G220" t="s">
+        <v>258</v>
+      </c>
+      <c r="H220" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="224" spans="3:8">
+      <c r="C224" s="10" t="s">
+        <v>254</v>
+      </c>
+      <c r="D224" s="10"/>
+    </row>
+    <row r="225" spans="3:8">
+      <c r="C225" t="s">
         <v>253</v>
       </c>
-      <c r="D220" t="s">
-        <v>254</v>
-      </c>
-      <c r="E220" t="s">
-        <v>255</v>
-      </c>
-      <c r="F220" t="s">
-        <v>256</v>
-      </c>
-      <c r="G220" t="s">
-        <v>257</v>
-      </c>
-      <c r="H220" t="s">
-        <v>258</v>
-      </c>
+      <c r="D225" t="s">
+        <v>228</v>
+      </c>
+      <c r="E225" t="s">
+        <v>10</v>
+      </c>
+      <c r="F225" t="s">
+        <v>79</v>
+      </c>
+      <c r="G225" t="s">
+        <v>78</v>
+      </c>
+      <c r="H225" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="226" spans="3:8">
+      <c r="C226" t="s">
+        <v>98</v>
+      </c>
+      <c r="D226">
+        <v>204.788738</v>
+      </c>
+      <c r="E226">
+        <v>10.400746</v>
+      </c>
+      <c r="F226">
+        <v>4.4748849999999996</v>
+      </c>
+      <c r="G226">
+        <v>5.9258610000000003</v>
+      </c>
+      <c r="H226">
+        <v>34.6537899428236</v>
+      </c>
+    </row>
+    <row r="227" spans="3:8">
+      <c r="C227" t="s">
+        <v>99</v>
+      </c>
+      <c r="D227">
+        <v>204.77824200000001</v>
+      </c>
+      <c r="E227">
+        <v>10.403459</v>
+      </c>
+      <c r="F227">
+        <v>4.4785029999999999</v>
+      </c>
+      <c r="G227">
+        <v>5.9249559999999999</v>
+      </c>
+      <c r="H227">
+        <v>34.658020764250601</v>
+      </c>
+    </row>
+    <row r="228" spans="3:8">
+      <c r="C228" t="s">
+        <v>241</v>
+      </c>
+      <c r="D228">
+        <v>204.78836100000001</v>
+      </c>
+      <c r="E228">
+        <v>10.399153</v>
+      </c>
+      <c r="F228">
+        <v>4.4735649999999998</v>
+      </c>
+      <c r="G228">
+        <v>5.9255880000000003</v>
+      </c>
+      <c r="H228">
+        <v>34.6558228237758</v>
+      </c>
+    </row>
+    <row r="229" spans="3:8">
+      <c r="C229" t="s">
+        <v>242</v>
+      </c>
+      <c r="D229">
+        <v>204.78702100000001</v>
+      </c>
+      <c r="E229">
+        <v>10.400496</v>
+      </c>
+      <c r="F229">
+        <v>4.475454</v>
+      </c>
+      <c r="G229">
+        <v>5.9250420000000004</v>
+      </c>
+      <c r="H229">
+        <v>34.658783185679901</v>
+      </c>
+    </row>
+    <row r="230" spans="3:8">
+      <c r="C230" t="s">
+        <v>243</v>
+      </c>
+      <c r="D230">
+        <v>204.77491499999999</v>
+      </c>
+      <c r="E230">
+        <v>10.398348</v>
+      </c>
+      <c r="F230">
+        <v>4.4729340000000004</v>
+      </c>
+      <c r="G230">
+        <v>5.925414</v>
+      </c>
+      <c r="H230">
+        <v>34.654721928537903</v>
+      </c>
+    </row>
+    <row r="231" spans="3:8">
+      <c r="C231" t="s">
+        <v>244</v>
+      </c>
+      <c r="D231">
+        <v>204.772796</v>
+      </c>
+      <c r="E231">
+        <v>10.399535999999999</v>
+      </c>
+      <c r="F231">
+        <v>4.4737539999999996</v>
+      </c>
+      <c r="G231">
+        <v>5.9257819999999999</v>
+      </c>
+      <c r="H231">
+        <v>34.651746302346901</v>
+      </c>
+    </row>
+    <row r="232" spans="3:8">
+      <c r="C232" t="s">
+        <v>245</v>
+      </c>
+      <c r="D232">
+        <v>204.781959</v>
+      </c>
+      <c r="E232">
+        <v>10.402101</v>
+      </c>
+      <c r="F232">
+        <v>4.4764470000000003</v>
+      </c>
+      <c r="G232">
+        <v>5.9256539999999998</v>
+      </c>
+      <c r="H232">
+        <v>34.653964935681898</v>
+      </c>
+    </row>
+    <row r="233" spans="3:8">
+      <c r="C233" t="s">
+        <v>246</v>
+      </c>
+      <c r="D233">
+        <v>204.770512</v>
+      </c>
+      <c r="E233">
+        <v>10.394026</v>
+      </c>
+      <c r="F233">
+        <v>4.4685329999999999</v>
+      </c>
+      <c r="G233">
+        <v>5.9254930000000003</v>
+      </c>
+      <c r="H233">
+        <v>34.653419221394998</v>
+      </c>
+    </row>
+    <row r="234" spans="3:8">
+      <c r="C234" t="s">
+        <v>247</v>
+      </c>
+      <c r="D234">
+        <v>204.781251</v>
+      </c>
+      <c r="E234">
+        <v>10.393862</v>
+      </c>
+      <c r="F234">
+        <v>4.4685740000000003</v>
+      </c>
+      <c r="G234">
+        <v>5.9252880000000001</v>
+      </c>
+      <c r="H234">
+        <v>34.656447302346898</v>
+      </c>
+    </row>
+    <row r="235" spans="3:8">
+      <c r="C235" t="s">
+        <v>248</v>
+      </c>
+      <c r="D235">
+        <v>204.783545</v>
+      </c>
+      <c r="E235">
+        <v>10.399879</v>
+      </c>
+      <c r="F235">
+        <v>4.4739589999999998</v>
+      </c>
+      <c r="G235">
+        <v>5.9259199999999996</v>
+      </c>
+      <c r="H235">
+        <v>34.652657592823203</v>
+      </c>
+    </row>
+    <row r="236" spans="3:8">
+      <c r="C236" t="s">
+        <v>249</v>
+      </c>
+      <c r="D236">
+        <f t="shared" ref="D236" si="4">AVERAGE(D226:D235)</f>
+        <v>204.780734</v>
+      </c>
+      <c r="E236">
+        <f>AVERAGE(E226:E235)</f>
+        <v>10.399160599999998</v>
+      </c>
+      <c r="F236">
+        <f t="shared" ref="F236" si="5">AVERAGE(F226:F235)</f>
+        <v>4.4736607999999993</v>
+      </c>
+      <c r="G236">
+        <f t="shared" ref="G236" si="6">AVERAGE(G226:G235)</f>
+        <v>5.9254998000000008</v>
+      </c>
+      <c r="H236">
+        <f t="shared" ref="H236" si="7">AVERAGE(H226:H235)</f>
+        <v>34.654937399966173</v>
+      </c>
+    </row>
+    <row r="237" spans="3:8">
+      <c r="C237" t="s">
+        <v>250</v>
+      </c>
+      <c r="D237">
+        <f t="shared" ref="D237" si="8">_xlfn.STDEV.S(D226:D235)</f>
+        <v>6.4893340010986319E-3</v>
+      </c>
+      <c r="E237">
+        <f>_xlfn.STDEV.S(E226:E235)</f>
+        <v>3.1122635635318593E-3</v>
+      </c>
+      <c r="F237">
+        <f t="shared" ref="F237:H237" si="9">_xlfn.STDEV.S(F226:F235)</f>
+        <v>3.1398679306973974E-3</v>
+      </c>
+      <c r="G237">
+        <f t="shared" si="9"/>
+        <v>3.2927421871604181E-4</v>
+      </c>
+      <c r="H237">
+        <f t="shared" si="9"/>
+        <v>2.2938382923205583E-3</v>
+      </c>
+    </row>
+    <row r="238" spans="3:8">
+      <c r="C238" t="s">
+        <v>251</v>
+      </c>
+      <c r="D238">
+        <f t="shared" ref="D238" si="10">_xlfn.CONFIDENCE.NORM(0.01,D237,COUNT(D226:D235))</f>
+        <v>5.2858788749296764E-3</v>
+      </c>
+      <c r="E238">
+        <f>_xlfn.CONFIDENCE.NORM(0.01,E237,COUNT(E226:E235))</f>
+        <v>2.5350903838361962E-3</v>
+      </c>
+      <c r="F238">
+        <f t="shared" ref="F238" si="11">_xlfn.CONFIDENCE.NORM(0.01,F237,COUNT(F226:F235))</f>
+        <v>2.5575754865033449E-3</v>
+      </c>
+      <c r="G238">
+        <f t="shared" ref="G238" si="12">_xlfn.CONFIDENCE.NORM(0.01,G237,COUNT(G226:G235))</f>
+        <v>2.6820990204471452E-4</v>
+      </c>
+      <c r="H238">
+        <f t="shared" ref="H238" si="13">_xlfn.CONFIDENCE.NORM(0.01,H237,COUNT(H226:H235))</f>
+        <v>1.8684431052291765E-3</v>
+      </c>
+    </row>
+    <row r="240" spans="3:8">
+      <c r="C240" t="s">
+        <v>252</v>
+      </c>
+      <c r="D240" t="s">
+        <v>260</v>
+      </c>
+      <c r="E240" t="s">
+        <v>264</v>
+      </c>
+      <c r="F240" t="s">
+        <v>261</v>
+      </c>
+      <c r="G240" t="s">
+        <v>262</v>
+      </c>
+      <c r="H240" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="243" spans="3:4">
+      <c r="C243" s="9" t="s">
+        <v>265</v>
+      </c>
+      <c r="D243" s="9"/>
+    </row>
+    <row r="244" spans="3:4" ht="15" customHeight="1">
+      <c r="C244" s="8" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="245" spans="3:4">
+      <c r="C245" s="8"/>
+    </row>
+    <row r="246" spans="3:4">
+      <c r="C246" s="8"/>
+    </row>
+    <row r="247" spans="3:4">
+      <c r="C247" s="8"/>
+    </row>
+    <row r="248" spans="3:4">
+      <c r="C248" s="8"/>
+    </row>
+    <row r="249" spans="3:4">
+      <c r="C249" s="8"/>
+    </row>
+    <row r="250" spans="3:4">
+      <c r="C250" s="8"/>
+    </row>
+    <row r="251" spans="3:4">
+      <c r="C251" s="8"/>
+    </row>
+    <row r="252" spans="3:4">
+      <c r="C252" s="8"/>
+    </row>
+    <row r="253" spans="3:4">
+      <c r="C253" s="8"/>
+    </row>
+    <row r="254" spans="3:4">
+      <c r="C254" s="8"/>
+    </row>
+    <row r="255" spans="3:4">
+      <c r="C255" s="8"/>
+    </row>
+    <row r="256" spans="3:4">
+      <c r="C256" s="8"/>
+    </row>
+    <row r="257" spans="3:3">
+      <c r="C257" s="8"/>
+    </row>
+    <row r="258" spans="3:3">
+      <c r="C258" s="8"/>
+    </row>
+    <row r="259" spans="3:3">
+      <c r="C259" s="8"/>
+    </row>
+    <row r="260" spans="3:3">
+      <c r="C260" s="8"/>
+    </row>
+    <row r="261" spans="3:3">
+      <c r="C261" s="8"/>
+    </row>
+    <row r="262" spans="3:3">
+      <c r="C262" s="8"/>
+    </row>
+    <row r="263" spans="3:3">
+      <c r="C263" s="8"/>
+    </row>
+    <row r="264" spans="3:3">
+      <c r="C264" s="8"/>
+    </row>
+    <row r="265" spans="3:3">
+      <c r="C265" s="8"/>
+    </row>
+    <row r="266" spans="3:3">
+      <c r="C266" s="8"/>
+    </row>
+    <row r="267" spans="3:3">
+      <c r="C267" s="8"/>
+    </row>
+    <row r="268" spans="3:3">
+      <c r="C268" s="8"/>
+    </row>
+    <row r="269" spans="3:3">
+      <c r="C269" s="8"/>
+    </row>
+    <row r="270" spans="3:3">
+      <c r="C270" s="8"/>
+    </row>
+    <row r="271" spans="3:3">
+      <c r="C271" s="8"/>
+    </row>
+    <row r="272" spans="3:3">
+      <c r="C272" s="8"/>
+    </row>
+    <row r="273" spans="3:3">
+      <c r="C273" s="8"/>
+    </row>
+    <row r="274" spans="3:3">
+      <c r="C274" s="13"/>
     </row>
   </sheetData>
   <autoFilter ref="C62:G62" xr:uid="{24461DB0-E066-4D80-9F31-EE0FB08E8CE2}">
@@ -9832,12 +11144,15 @@
       <sortCondition descending="1" ref="F62"/>
     </sortState>
   </autoFilter>
-  <mergeCells count="5">
+  <mergeCells count="8">
+    <mergeCell ref="C28:C59"/>
+    <mergeCell ref="I63:I69"/>
+    <mergeCell ref="C244:C273"/>
+    <mergeCell ref="I174:I183"/>
+    <mergeCell ref="C243:D243"/>
+    <mergeCell ref="C224:D224"/>
     <mergeCell ref="C113:C170"/>
     <mergeCell ref="C92:C110"/>
-    <mergeCell ref="C28:C59"/>
-    <mergeCell ref="I63:I69"/>
-    <mergeCell ref="J174:J183"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <conditionalFormatting sqref="D63:D81">
@@ -45195,13 +46510,13 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24B647F8-E4E5-49C3-B391-C8FB35E3608C}">
-  <dimension ref="B2:W13"/>
+  <dimension ref="B2:AK13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="12.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:23">
+    <row r="2" spans="2:37">
       <c r="B2" t="s">
         <v>16</v>
       </c>
@@ -45251,22 +46566,64 @@
         <v>42</v>
       </c>
       <c r="S2" t="s">
+        <v>72</v>
+      </c>
+      <c r="T2" t="s">
+        <v>73</v>
+      </c>
+      <c r="U2" t="s">
+        <v>74</v>
+      </c>
+      <c r="V2" t="s">
+        <v>75</v>
+      </c>
+      <c r="W2" t="s">
+        <v>76</v>
+      </c>
+      <c r="X2" t="s">
+        <v>80</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>81</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>82</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>83</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>84</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>85</v>
+      </c>
+      <c r="AD2" t="s">
+        <v>86</v>
+      </c>
+      <c r="AE2" t="s">
+        <v>87</v>
+      </c>
+      <c r="AF2" t="s">
+        <v>88</v>
+      </c>
+      <c r="AG2" t="s">
         <v>50</v>
       </c>
-      <c r="T2" t="s">
+      <c r="AH2" t="s">
         <v>49</v>
       </c>
-      <c r="U2" t="s">
+      <c r="AI2" t="s">
         <v>48</v>
       </c>
-      <c r="V2" t="s">
+      <c r="AJ2" t="s">
         <v>51</v>
       </c>
-      <c r="W2" t="s">
+      <c r="AK2" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="3" spans="2:23">
+    <row r="3" spans="2:37">
       <c r="C3" t="s">
         <v>18</v>
       </c>
@@ -45285,28 +46642,42 @@
       <c r="P3" s="1"/>
       <c r="Q3" s="1"/>
       <c r="R3" s="1"/>
-      <c r="S3">
+      <c r="S3" s="1"/>
+      <c r="T3" s="1"/>
+      <c r="U3" s="1"/>
+      <c r="V3" s="1"/>
+      <c r="W3" s="1"/>
+      <c r="X3" s="1"/>
+      <c r="Y3" s="1"/>
+      <c r="Z3" s="1"/>
+      <c r="AA3" s="1"/>
+      <c r="AB3" s="1"/>
+      <c r="AC3" s="1"/>
+      <c r="AD3" s="1"/>
+      <c r="AE3" s="1"/>
+      <c r="AF3" s="1"/>
+      <c r="AG3">
         <f>SUM(D3:R3)</f>
         <v>0</v>
       </c>
-      <c r="T3">
+      <c r="AH3">
         <f>COUNT(D3:R3)</f>
         <v>0</v>
       </c>
-      <c r="U3">
+      <c r="AI3">
         <f>COUNTIF(D3:R3,0)</f>
         <v>0</v>
       </c>
-      <c r="V3">
-        <f>T3-U3</f>
-        <v>0</v>
-      </c>
-      <c r="W3" t="e">
-        <f>S3/V3</f>
+      <c r="AJ3">
+        <f>AH3-AI3</f>
+        <v>0</v>
+      </c>
+      <c r="AK3" t="e">
+        <f>AG3/AJ3</f>
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="4" spans="2:23">
+    <row r="4" spans="2:37">
       <c r="C4" t="s">
         <v>31</v>
       </c>
@@ -45325,28 +46696,42 @@
       <c r="P4" s="1"/>
       <c r="Q4" s="1"/>
       <c r="R4" s="1"/>
-      <c r="S4">
-        <f t="shared" ref="S4:S12" si="0">SUM(D4:R4)</f>
-        <v>0</v>
-      </c>
-      <c r="T4">
-        <f t="shared" ref="T4:T12" si="1">COUNT(D4:R4)</f>
-        <v>0</v>
-      </c>
-      <c r="U4">
-        <f t="shared" ref="U4:U12" si="2">COUNTIF(D4:R4,0)</f>
-        <v>0</v>
-      </c>
-      <c r="V4">
-        <f t="shared" ref="V4:V12" si="3">T4-U4</f>
-        <v>0</v>
-      </c>
-      <c r="W4" t="e">
-        <f t="shared" ref="W4:W12" si="4">S4/V4</f>
+      <c r="S4" s="1"/>
+      <c r="T4" s="1"/>
+      <c r="U4" s="1"/>
+      <c r="V4" s="1"/>
+      <c r="W4" s="1"/>
+      <c r="X4" s="1"/>
+      <c r="Y4" s="1"/>
+      <c r="Z4" s="1"/>
+      <c r="AA4" s="1"/>
+      <c r="AB4" s="1"/>
+      <c r="AC4" s="1"/>
+      <c r="AD4" s="1"/>
+      <c r="AE4" s="1"/>
+      <c r="AF4" s="1"/>
+      <c r="AG4">
+        <f>SUM(D4:R4)</f>
+        <v>0</v>
+      </c>
+      <c r="AH4">
+        <f>COUNT(D4:R4)</f>
+        <v>0</v>
+      </c>
+      <c r="AI4">
+        <f>COUNTIF(D4:R4,0)</f>
+        <v>0</v>
+      </c>
+      <c r="AJ4">
+        <f t="shared" ref="AJ4:AJ12" si="0">AH4-AI4</f>
+        <v>0</v>
+      </c>
+      <c r="AK4" t="e">
+        <f t="shared" ref="AK4:AK12" si="1">AG4/AJ4</f>
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="5" spans="2:23">
+    <row r="5" spans="2:37">
       <c r="C5" t="s">
         <v>32</v>
       </c>
@@ -45365,28 +46750,42 @@
       <c r="P5" s="1"/>
       <c r="Q5" s="1"/>
       <c r="R5" s="1"/>
-      <c r="S5">
+      <c r="S5" s="1"/>
+      <c r="T5" s="1"/>
+      <c r="U5" s="1"/>
+      <c r="V5" s="1"/>
+      <c r="W5" s="1"/>
+      <c r="X5" s="1"/>
+      <c r="Y5" s="1"/>
+      <c r="Z5" s="1"/>
+      <c r="AA5" s="1"/>
+      <c r="AB5" s="1"/>
+      <c r="AC5" s="1"/>
+      <c r="AD5" s="1"/>
+      <c r="AE5" s="1"/>
+      <c r="AF5" s="1"/>
+      <c r="AG5">
+        <f>SUM(D5:R5)</f>
+        <v>0</v>
+      </c>
+      <c r="AH5">
+        <f>COUNT(D5:R5)</f>
+        <v>0</v>
+      </c>
+      <c r="AI5">
+        <f>COUNTIF(D5:R5,0)</f>
+        <v>0</v>
+      </c>
+      <c r="AJ5">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="T5">
+      <c r="AK5" t="e">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="U5">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="V5">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="W5" t="e">
-        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="6" spans="2:23">
+    <row r="6" spans="2:37">
       <c r="C6" t="s">
         <v>33</v>
       </c>
@@ -45405,28 +46804,42 @@
       <c r="P6" s="1"/>
       <c r="Q6" s="1"/>
       <c r="R6" s="1"/>
-      <c r="S6">
+      <c r="S6" s="1"/>
+      <c r="T6" s="1"/>
+      <c r="U6" s="1"/>
+      <c r="V6" s="1"/>
+      <c r="W6" s="1"/>
+      <c r="X6" s="1"/>
+      <c r="Y6" s="1"/>
+      <c r="Z6" s="1"/>
+      <c r="AA6" s="1"/>
+      <c r="AB6" s="1"/>
+      <c r="AC6" s="1"/>
+      <c r="AD6" s="1"/>
+      <c r="AE6" s="1"/>
+      <c r="AF6" s="1"/>
+      <c r="AG6">
+        <f>SUM(D6:R6)</f>
+        <v>0</v>
+      </c>
+      <c r="AH6">
+        <f>COUNT(D6:R6)</f>
+        <v>0</v>
+      </c>
+      <c r="AI6">
+        <f>COUNTIF(D6:R6,0)</f>
+        <v>0</v>
+      </c>
+      <c r="AJ6">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="T6">
+      <c r="AK6" t="e">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="U6">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="V6">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="W6" t="e">
-        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="7" spans="2:23">
+    <row r="7" spans="2:37">
       <c r="C7" t="s">
         <v>34</v>
       </c>
@@ -45445,28 +46858,42 @@
       <c r="P7" s="1"/>
       <c r="Q7" s="1"/>
       <c r="R7" s="1"/>
-      <c r="S7">
+      <c r="S7" s="1"/>
+      <c r="T7" s="1"/>
+      <c r="U7" s="1"/>
+      <c r="V7" s="1"/>
+      <c r="W7" s="1"/>
+      <c r="X7" s="1"/>
+      <c r="Y7" s="1"/>
+      <c r="Z7" s="1"/>
+      <c r="AA7" s="1"/>
+      <c r="AB7" s="1"/>
+      <c r="AC7" s="1"/>
+      <c r="AD7" s="1"/>
+      <c r="AE7" s="1"/>
+      <c r="AF7" s="1"/>
+      <c r="AG7">
+        <f>SUM(D7:R7)</f>
+        <v>0</v>
+      </c>
+      <c r="AH7">
+        <f>COUNT(D7:R7)</f>
+        <v>0</v>
+      </c>
+      <c r="AI7">
+        <f>COUNTIF(D7:R7,0)</f>
+        <v>0</v>
+      </c>
+      <c r="AJ7">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="T7">
+      <c r="AK7" t="e">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="U7">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="V7">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="W7" t="e">
-        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="8" spans="2:23">
+    <row r="8" spans="2:37">
       <c r="C8" t="s">
         <v>35</v>
       </c>
@@ -45485,28 +46912,42 @@
       <c r="P8" s="1"/>
       <c r="Q8" s="1"/>
       <c r="R8" s="1"/>
-      <c r="S8">
+      <c r="S8" s="1"/>
+      <c r="T8" s="1"/>
+      <c r="U8" s="1"/>
+      <c r="V8" s="1"/>
+      <c r="W8" s="1"/>
+      <c r="X8" s="1"/>
+      <c r="Y8" s="1"/>
+      <c r="Z8" s="1"/>
+      <c r="AA8" s="1"/>
+      <c r="AB8" s="1"/>
+      <c r="AC8" s="1"/>
+      <c r="AD8" s="1"/>
+      <c r="AE8" s="1"/>
+      <c r="AF8" s="1"/>
+      <c r="AG8">
+        <f>SUM(D8:R8)</f>
+        <v>0</v>
+      </c>
+      <c r="AH8">
+        <f>COUNT(D8:R8)</f>
+        <v>0</v>
+      </c>
+      <c r="AI8">
+        <f>COUNTIF(D8:R8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="AJ8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="T8">
+      <c r="AK8" t="e">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="U8">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="V8">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="W8" t="e">
-        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="9" spans="2:23">
+    <row r="9" spans="2:37">
       <c r="C9" t="s">
         <v>36</v>
       </c>
@@ -45525,28 +46966,42 @@
       <c r="P9" s="1"/>
       <c r="Q9" s="1"/>
       <c r="R9" s="1"/>
-      <c r="S9">
+      <c r="S9" s="1"/>
+      <c r="T9" s="1"/>
+      <c r="U9" s="1"/>
+      <c r="V9" s="1"/>
+      <c r="W9" s="1"/>
+      <c r="X9" s="1"/>
+      <c r="Y9" s="1"/>
+      <c r="Z9" s="1"/>
+      <c r="AA9" s="1"/>
+      <c r="AB9" s="1"/>
+      <c r="AC9" s="1"/>
+      <c r="AD9" s="1"/>
+      <c r="AE9" s="1"/>
+      <c r="AF9" s="1"/>
+      <c r="AG9">
+        <f>SUM(D9:R9)</f>
+        <v>0</v>
+      </c>
+      <c r="AH9">
+        <f>COUNT(D9:R9)</f>
+        <v>0</v>
+      </c>
+      <c r="AI9">
+        <f>COUNTIF(D9:R9,0)</f>
+        <v>0</v>
+      </c>
+      <c r="AJ9">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="T9">
+      <c r="AK9" t="e">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="U9">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="V9">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="W9" t="e">
-        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="10" spans="2:23">
+    <row r="10" spans="2:37">
       <c r="C10" t="s">
         <v>37</v>
       </c>
@@ -45565,28 +47020,42 @@
       <c r="P10" s="1"/>
       <c r="Q10" s="1"/>
       <c r="R10" s="1"/>
-      <c r="S10">
+      <c r="S10" s="1"/>
+      <c r="T10" s="1"/>
+      <c r="U10" s="1"/>
+      <c r="V10" s="1"/>
+      <c r="W10" s="1"/>
+      <c r="X10" s="1"/>
+      <c r="Y10" s="1"/>
+      <c r="Z10" s="1"/>
+      <c r="AA10" s="1"/>
+      <c r="AB10" s="1"/>
+      <c r="AC10" s="1"/>
+      <c r="AD10" s="1"/>
+      <c r="AE10" s="1"/>
+      <c r="AF10" s="1"/>
+      <c r="AG10">
+        <f>SUM(D10:R10)</f>
+        <v>0</v>
+      </c>
+      <c r="AH10">
+        <f>COUNT(D10:R10)</f>
+        <v>0</v>
+      </c>
+      <c r="AI10">
+        <f>COUNTIF(D10:R10,0)</f>
+        <v>0</v>
+      </c>
+      <c r="AJ10">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="T10">
+      <c r="AK10" t="e">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="U10">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="V10">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="W10" t="e">
-        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="11" spans="2:23">
+    <row r="11" spans="2:37">
       <c r="C11" t="s">
         <v>38</v>
       </c>
@@ -45605,28 +47074,42 @@
       <c r="P11" s="1"/>
       <c r="Q11" s="1"/>
       <c r="R11" s="1"/>
-      <c r="S11">
+      <c r="S11" s="1"/>
+      <c r="T11" s="1"/>
+      <c r="U11" s="1"/>
+      <c r="V11" s="1"/>
+      <c r="W11" s="1"/>
+      <c r="X11" s="1"/>
+      <c r="Y11" s="1"/>
+      <c r="Z11" s="1"/>
+      <c r="AA11" s="1"/>
+      <c r="AB11" s="1"/>
+      <c r="AC11" s="1"/>
+      <c r="AD11" s="1"/>
+      <c r="AE11" s="1"/>
+      <c r="AF11" s="1"/>
+      <c r="AG11">
+        <f>SUM(D11:R11)</f>
+        <v>0</v>
+      </c>
+      <c r="AH11">
+        <f>COUNT(D11:R11)</f>
+        <v>0</v>
+      </c>
+      <c r="AI11">
+        <f>COUNTIF(D11:R11,0)</f>
+        <v>0</v>
+      </c>
+      <c r="AJ11">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="T11">
+      <c r="AK11" t="e">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="U11">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="V11">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="W11" t="e">
-        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="12" spans="2:23">
+    <row r="12" spans="2:37">
       <c r="C12" t="s">
         <v>39</v>
       </c>
@@ -45645,50 +47128,65 @@
       <c r="P12" s="1"/>
       <c r="Q12" s="1"/>
       <c r="R12" s="1"/>
-      <c r="S12">
+      <c r="S12" s="1"/>
+      <c r="T12" s="1"/>
+      <c r="U12" s="1"/>
+      <c r="V12" s="1"/>
+      <c r="W12" s="1"/>
+      <c r="X12" s="1"/>
+      <c r="Y12" s="1"/>
+      <c r="Z12" s="1"/>
+      <c r="AA12" s="1"/>
+      <c r="AB12" s="1"/>
+      <c r="AC12" s="1"/>
+      <c r="AD12" s="1"/>
+      <c r="AE12" s="1"/>
+      <c r="AF12" s="1"/>
+      <c r="AG12">
+        <f>SUM(D12:R12)</f>
+        <v>0</v>
+      </c>
+      <c r="AH12">
+        <f>COUNT(D12:R12)</f>
+        <v>0</v>
+      </c>
+      <c r="AI12">
+        <f>COUNTIF(D12:R12,0)</f>
+        <v>0</v>
+      </c>
+      <c r="AJ12">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="T12">
+      <c r="AK12" t="e">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="U12">
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="13" spans="2:37">
+      <c r="AG13" t="s">
+        <v>52</v>
+      </c>
+      <c r="AH13">
+        <f>AVERAGE(AH3:AH12)</f>
+        <v>0</v>
+      </c>
+      <c r="AI13">
+        <f t="shared" ref="AI13:AK13" si="2">AVERAGE(AI3:AI12)</f>
+        <v>0</v>
+      </c>
+      <c r="AJ13">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="V12">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="W12" t="e">
-        <f t="shared" si="4"/>
+      <c r="AK13" t="e">
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="13" spans="2:23">
-      <c r="S13" t="s">
-        <v>52</v>
-      </c>
-      <c r="T13">
-        <f>AVERAGE(T3:T12)</f>
-        <v>0</v>
-      </c>
-      <c r="U13">
-        <f t="shared" ref="U13:W13" si="5">AVERAGE(U3:U12)</f>
-        <v>0</v>
-      </c>
-      <c r="V13">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="W13" t="e">
-        <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="D3:R12">
+  <phoneticPr fontId="3" type="noConversion"/>
+  <conditionalFormatting sqref="D3:AF12">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>